<commit_message>
Align worksheet guide with final catalog
</commit_message>
<xml_diff>
--- a/EEG_healthcare_disease_catalog_20260823.xlsx
+++ b/EEG_healthcare_disease_catalog_20260823.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R9874b7a91dfc4a81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最终唯一下载清单" sheetId="2" r:id="Rfd2e7fccdf504142"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="排除与非独立条目" sheetId="3" r:id="R02cd2ad17bf144e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="重复合并证据" sheetId="4" r:id="R73ff9d2d59b542f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人工复核结论" sheetId="5" r:id="Rcda4969dd6c5457d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TUH体系与重叠" sheetId="6" r:id="Ra12ffd0c4b604344"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="文件夹架构" sheetId="7" r:id="R2adf23849fef46e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="修订记录" sheetId="8" r:id="R49318283a86c4310"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原重复证据归档" sheetId="9" r:id="R34c92b984a664bb6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类复核" sheetId="12" r:id="Rd8c205b50574489d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类修订明细" sheetId="13" r:id="R5ec5704ffb384a90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="下载与时长复核" sheetId="14" r:id="Red4056264e134be4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="证据来源" sheetId="15" r:id="Rea858dfc4d7e47d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Healthcare重点清单" sheetId="16" r:id="Raaa4a49b944343b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增来源记录_25" sheetId="17" r:id="Rc5b2cec2f7894485"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类统计" sheetId="18" r:id="Rff6c8dbfb66c416a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REVE对照_92" sheetId="19" r:id="R41ff64739a2542d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NeuroAtlas对照_42" sheetId="20" r:id="R66ec58e9474d4920"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R410e0069897c4ae0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最终唯一下载清单" sheetId="2" r:id="R83bab91c195b4f59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="排除与非独立条目" sheetId="3" r:id="R24b97b71340a48b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="重复合并证据" sheetId="4" r:id="R8d6aa8bdb0214caa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人工复核结论" sheetId="5" r:id="Rc81091a8f0114996"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TUH体系与重叠" sheetId="6" r:id="Rfbfc71c6577c4c8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="文件夹架构" sheetId="7" r:id="Rd25076f4a29f4b80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="修订记录" sheetId="8" r:id="R09ca16e63f3047cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原重复证据归档" sheetId="9" r:id="R3b559022ee7945b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类复核" sheetId="12" r:id="R4a05d9cc22cd411a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类修订明细" sheetId="13" r:id="Rff606295f9404cd5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="下载与时长复核" sheetId="14" r:id="R2b7588b488ee4906"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="证据来源" sheetId="15" r:id="R5682c3f1e5a04ae4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Healthcare重点清单" sheetId="16" r:id="Rac07c3f1c15a4895"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增来源记录_25" sheetId="17" r:id="R457fea0ed42d4f4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类统计" sheetId="18" r:id="R37be12be00f34cd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REVE对照_92" sheetId="19" r:id="R491fe204265a4975"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NeuroAtlas对照_42" sheetId="20" r:id="Rdc4e7a03bc724719"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2241,7 +2241,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14e70600e8cb41ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89a92d2c78084130"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4810,7 +4810,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5a71e25bb3649e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2313481f88284b10"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6882,7 +6882,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60fcffefa7844a54"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4adaebfff9ff4589"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7119,7 +7119,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5615865a88fb4c09"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9f61a363d614d3c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13149,7 +13149,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2d7a964af124952"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c5cb0fd919d4a95"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14794,7 +14794,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb53b9235999e4323"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40064723c6f0469c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15686,7 +15686,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rafcbbfc7b3d64e02"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R583bdbeb7e5245b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17191,8 +17191,8 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e8d6dc460f740e2"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3b139c5e50a4d91"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd85f46470174fd2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb15ba0696d9c46b9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18536,7 +18536,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc61d20ec57042b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5cb63b835664410"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -50601,7 +50601,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce71e8010bb44288"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8fbc6ca6bac4336"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -53115,7 +53115,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1266d10a26004006"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re01dc71710e1464f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -54333,7 +54333,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6e769c141ea42b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R182c26b556214e8d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -54513,7 +54513,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7efd5f7fa5704b5e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref55144fb6614e9b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -54818,7 +54818,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd36c6575a2de4c57"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61abd25557554270"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -55591,7 +55591,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4548940fae814d62"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab997bd1b0f846ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -55791,7 +55791,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra501ecd16cac436f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6cdcd1de2524f17"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -57533,7 +57533,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R944c5d249f084e1d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raaec24227f6d46d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update subject totals and authorized download status
</commit_message>
<xml_diff>
--- a/EEG_healthcare_disease_catalog_20260823.xlsx
+++ b/EEG_healthcare_disease_catalog_20260823.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R3f14c6a282854b1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最终唯一下载清单" sheetId="2" r:id="Rd1e174399cc143cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="修订记录" sheetId="8" r:id="R469bf10cea8945db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R7cc5c9c0f93141e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最终唯一下载清单" sheetId="2" r:id="R023ca09c7b3b4aa8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="修订记录" sheetId="8" r:id="R3e080f1b493c4c6a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1580,7 +1580,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="RevisionLog20260823" displayName="RevisionLog20260823" ref="A1:F11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="RevisionLog20260823" displayName="RevisionLog20260823" ref="A1:F13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Change type"/>
@@ -1883,7 +1883,7 @@
         <x:v>正式申请</x:v>
       </x:c>
       <x:c r="B12" s="213" t="str">
-        <x:v>43 个：21 个已申请等待，22 个尚需提交</x:v>
+        <x:v>41 个：19 个已申请等待，22 个尚需提交</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="58" customHeight="1">
@@ -1891,7 +1891,7 @@
         <x:v>直接推进</x:v>
       </x:c>
       <x:c r="B13" s="213" t="str">
-        <x:v>19 个可直接下载；1 个只需登录；5 个需人工确认文件入口</x:v>
+        <x:v>19 个可直接下载；2 个只需登录；6 个需人工确认文件入口</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="58" customHeight="1">
@@ -1987,22 +1987,38 @@
         <x:v>受试者口径</x:v>
       </x:c>
       <x:c r="B25" s="215" t="str">
-        <x:v>94,700 dataset-subject entries（来源行合计；不是跨数据集去重后的唯一人数）</x:v>
+        <x:v>99,515 dataset-subject entries（来源行合计；不是跨数据集去重后的唯一人数）</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="243" t="str">
+        <x:v>已获批访问</x:v>
+      </x:c>
+      <x:c r="B26" s="215" t="str">
+        <x:v>CHBMP：32/250 raw sessions 已下载并审计 10.9689 h；MODMA：ID 13/14/17 已获批，但官网当前不可达。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="243" t="str">
+        <x:v>MESA 申请</x:v>
+      </x:c>
+      <x:c r="B27" s="215" t="str">
+        <x:v>申请标准 MESA Sleep（raw PSG EDF + XML annotations + 核心协变量），不是 MESA-COMMERCIAL-USE；raw PSG/EEG 为 2,056 名参与者。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="243" t="str">
         <x:v>推荐阅读</x:v>
       </x:c>
-      <x:c r="B26" s="215" t="str">
+      <x:c r="B28" s="215" t="str">
         <x:v>README → 最终唯一下载清单 → 修订记录</x:v>
       </x:c>
     </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="245" t="str">
+    <x:row r="29">
+      <x:c r="A29" s="245" t="str">
         <x:v>谨慎原则</x:v>
       </x:c>
-      <x:c r="B27" s="228" t="str">
+      <x:c r="B29" s="228" t="str">
         <x:v>未知总时长保持空白，不用 8 h/晚等假设制造精确感。</x:v>
       </x:c>
     </x:row>
@@ -6207,7 +6223,7 @@
         <x:v>03_Consciousness_and_State/Sleep_Staging/DREAMER</x:v>
       </x:c>
       <x:c r="R71" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号 分类复核：DREAMER is an affective EEG/ECG experiment, not a sleep-health dataset.</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 分类复核：DREAMER is an affective EEG/ECG experiment, not a sleep-health dataset. 分类复核：DREAMER is an affective EEG/ECG experiment, not a sleep-health dataset.</x:v>
       </x:c>
       <x:c r="S71" s="257"/>
       <x:c r="T71" s="257"/>
@@ -6230,13 +6246,13 @@
         <x:v>Dreem Open Datasets; DOD-H/DOD-O</x:v>
       </x:c>
       <x:c r="F72" s="275" t="str">
-        <x:v>Dreem official S3:DOD-H | GitHub:Dreem-Organization/dreem-learning-open</x:v>
+        <x:v>DOI:10.5281/zenodo.15900394 | GitHub:Dreem-Organization/dreem-learning-open</x:v>
       </x:c>
       <x:c r="G72" s="275" t="str">
         <x:v>DOWNLOAD_PUBLIC</x:v>
       </x:c>
       <x:c r="H72" s="275" t="str">
-        <x:v>https://dreem-dodo-dodh.s3.eu-west-1.amazonaws.com/index.html</x:v>
+        <x:v>https://zenodo.org/records/15900394</x:v>
       </x:c>
       <x:c r="I72" s="275" t="str">
         <x:v>Sleep staging with clinical PSG and wearable headband</x:v>
@@ -6266,7 +6282,7 @@
         <x:v>03_Consciousness_and_State/Sleep_Staging/Dreem_Open_Datasets_DOD-H</x:v>
       </x:c>
       <x:c r="R72" s="275" t="str">
-        <x:v>官方 S3 提供公开下载；原 Zenodo:4498364 实为无关的 COUGHVID 记录，已纠正。</x:v>
+        <x:v>Dreem 官方仓库现指向 Zenodo:15900394；DOD-H 为 dodh.zip（21.9 GB）。旧 S3 桶已不存在，已更正入口。</x:v>
       </x:c>
       <x:c r="S72" s="275"/>
       <x:c r="T72" s="275"/>
@@ -6553,7 +6569,7 @@
         <x:v>03_Consciousness_and_State/Sleep_Staging/MAHNOB-HCI</x:v>
       </x:c>
       <x:c r="R77" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号；2026-08-04去重：EEG-0184并入EEG-0129（MAHNOB-HCI official database identity） 分类复核：MAHNOB-HCI is multimodal affect recognition, not sleep staging.</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号；2026-08-04去重：EEG-0184并入EEG-0129（MAHNOB-HCI official database identity） 分类复核：MAHNOB-HCI is multimodal affect recognition, not sleep staging. 分类复核：MAHNOB-HCI is multimodal affect recognition, not sleep staging.</x:v>
       </x:c>
       <x:c r="S77" s="257"/>
       <x:c r="T77" s="257"/>
@@ -6961,7 +6977,7 @@
         <x:v>03_Consciousness_and_State/Sleep_Staging/Test-Retest_RestCog</x:v>
       </x:c>
       <x:c r="R84" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号 分类复核：RestCog is a healthy rest/cognitive-state benchmark, not a disease or population-health cohort.</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 分类复核：RestCog is a healthy rest/cognitive-state benchmark, not a disease or population-health cohort. 分类复核：RestCog is a healthy rest/cognitive-state benchmark, not a disease or population-health cohort.</x:v>
       </x:c>
       <x:c r="S84" s="275"/>
       <x:c r="T84" s="275"/>
@@ -33258,7 +33274,7 @@
         <x:v>03_Consciousness_and_State/Sleep_Staging/ASCERTAIN</x:v>
       </x:c>
       <x:c r="R548" s="280" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号 分类复核：ASCERTAIN is an affect/personality experiment, not a sleep or clinical cohort.</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 分类复核：ASCERTAIN is an affect/personality experiment, not a sleep or clinical cohort. 分类复核：ASCERTAIN is an affect/personality experiment, not a sleep or clinical cohort.</x:v>
       </x:c>
       <x:c r="S548" s="280"/>
       <x:c r="T548" s="280"/>
@@ -34074,7 +34090,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3126b06677354cdd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R900dd76072214f62"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34242,10 +34258,10 @@
         <x:v>EEG-0093 / EEG-0122</x:v>
       </x:c>
       <x:c r="D8" s="400" t="str">
-        <x:v>PD-Mortality 更新为 OpenNeuro ds007020 公开下载；DOD-H 改为官方 S3，删除错误 Zenodo:4498364。</x:v>
+        <x:v>PD-Mortality 更新为 OpenNeuro ds007020 公开下载；DOD-H 更新为官方 Zenodo:15900394。</x:v>
       </x:c>
       <x:c r="E8" s="400" t="str">
-        <x:v>OpenNeuro/NEMAR；Dreem official S3/GitHub</x:v>
+        <x:v>OpenNeuro ds007020；DOI:10.5281/zenodo.15900394</x:v>
       </x:c>
       <x:c r="F8" s="401" t="str">
         <x:v>转为直接下载</x:v>
@@ -34259,16 +34275,16 @@
         <x:v>ACCESS</x:v>
       </x:c>
       <x:c r="C9" s="257" t="str">
-        <x:v>MORGOTH PSG</x:v>
+        <x:v>MODMA / CHBMP</x:v>
       </x:c>
       <x:c r="D9" s="257" t="str">
-        <x:v>4 个 PSG 子集并入已提交的 MORGOTH credentialed-access 申请。</x:v>
+        <x:v>MODMA ID 13/14/17 已获批但官网当前不可达；CHBMP 已获批，首批 32/250 raw sessions 下载并完成 EDF 头审计。</x:v>
       </x:c>
       <x:c r="E9" s="257" t="str">
-        <x:v>BDSP MORGOTH 1.0</x:v>
+        <x:v>MODMA 个人授权；CHBMP LORIS</x:v>
       </x:c>
       <x:c r="F9" s="213" t="str">
-        <x:v>等待授权</x:v>
+        <x:v>CHBMP 新增 32 EDF / 10.9689 h</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -34276,45 +34292,85 @@
         <x:v>2026-08-23</x:v>
       </x:c>
       <x:c r="B10" s="328" t="str">
+        <x:v>DOWNLOAD</x:v>
+      </x:c>
+      <x:c r="C10" s="328" t="str">
+        <x:v>19 public units</x:v>
+      </x:c>
+      <x:c r="D10" s="328" t="str">
+        <x:v>19 个直下单元总量超过当前 2.8 TB 空闲；先启动 EEG-Bench 4 项、PD-Mortality、DOD-H、HMC、UCDDB。</x:v>
+      </x:c>
+      <x:c r="E10" s="328" t="str">
+        <x:v>官方对象大小与服务器 df 审计</x:v>
+      </x:c>
+      <x:c r="F10" s="329" t="str">
+        <x:v>Slurm 2133731</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="226" t="str">
+        <x:v>2026-08-23</x:v>
+      </x:c>
+      <x:c r="B11" s="259" t="str">
+        <x:v>ACCESS</x:v>
+      </x:c>
+      <x:c r="C11" s="259" t="str">
+        <x:v>MORGOTH PSG</x:v>
+      </x:c>
+      <x:c r="D11" s="259" t="str">
+        <x:v>4 个 PSG 子集并入已提交的 MORGOTH credentialed-access 申请。</x:v>
+      </x:c>
+      <x:c r="E11" s="259" t="str">
+        <x:v>BDSP MORGOTH 1.0</x:v>
+      </x:c>
+      <x:c r="F11" s="215" t="str">
+        <x:v>等待授权</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="233" t="str">
+        <x:v>2026-08-23</x:v>
+      </x:c>
+      <x:c r="B12" s="328" t="str">
         <x:v>QUEUE</x:v>
       </x:c>
-      <x:c r="C10" s="328" t="str">
+      <x:c r="C12" s="328" t="str">
         <x:v>68 actionable</x:v>
       </x:c>
-      <x:c r="D10" s="328" t="str">
-        <x:v>正式需申请 43 项：已申请 21 项，尚需申请 22 项；另有 4 项舍弃。</x:v>
-      </x:c>
-      <x:c r="E10" s="328" t="str">
+      <x:c r="D12" s="328" t="str">
+        <x:v>正式需申请 41 项：已申请 19 项，尚需申请 22 项；另有 4 项舍弃。</x:v>
+      </x:c>
+      <x:c r="E12" s="328" t="str">
         <x:v>逐项官方访问入口复核</x:v>
       </x:c>
-      <x:c r="F10" s="329" t="str">
+      <x:c r="F12" s="329" t="str">
         <x:v>更新执行队列</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="227" t="str">
+    <x:row r="13">
+      <x:c r="A13" s="227" t="str">
         <x:v>2026-08-23</x:v>
       </x:c>
-      <x:c r="B11" s="270" t="str">
+      <x:c r="B13" s="270" t="str">
         <x:v>FORMAT</x:v>
       </x:c>
-      <x:c r="C11" s="270" t="str">
+      <x:c r="C13" s="270" t="str">
         <x:v>Workbook</x:v>
       </x:c>
-      <x:c r="D11" s="270" t="str">
+      <x:c r="D13" s="270" t="str">
         <x:v>公开下载工作簿精简为 README、最终唯一下载清单、修订记录 3 张表。</x:v>
       </x:c>
-      <x:c r="E11" s="270" t="str">
+      <x:c r="E13" s="270" t="str">
         <x:v>用户要求</x:v>
       </x:c>
-      <x:c r="F11" s="228" t="str">
+      <x:c r="F13" s="228" t="str">
         <x:v>无</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e5fd63bd07c4219"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76b0eaeb1acf4c0c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Mark MODMA approved login access
</commit_message>
<xml_diff>
--- a/EEG_healthcare_disease_catalog_20260823.xlsx
+++ b/EEG_healthcare_disease_catalog_20260823.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R7cc5c9c0f93141e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最终唯一下载清单" sheetId="2" r:id="R023ca09c7b3b4aa8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="修订记录" sheetId="8" r:id="R3e080f1b493c4c6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R3fd9d4fe936b4764"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最终唯一下载清单" sheetId="2" r:id="R59a635ffaf1a4ba5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="修订记录" sheetId="8" r:id="Rb4dcd415287a4db9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1891,7 +1891,7 @@
         <x:v>直接推进</x:v>
       </x:c>
       <x:c r="B13" s="213" t="str">
-        <x:v>19 个可直接下载；2 个只需登录；6 个需人工确认文件入口</x:v>
+        <x:v>19 个可直接下载；3 个只需登录；5 个需人工确认文件入口</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="58" customHeight="1">
@@ -1995,7 +1995,7 @@
         <x:v>已获批访问</x:v>
       </x:c>
       <x:c r="B26" s="215" t="str">
-        <x:v>CHBMP：32/250 raw sessions 已下载并审计 10.9689 h；MODMA：ID 13/14/17 已获批，但官网当前不可达。</x:v>
+        <x:v>CHBMP：32/250 raw sessions 已下载并审计 10.9689 h；MODMA：ID 13/14/17 已获批，入口双端复测恢复，需重新登录。</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -34090,7 +34090,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R900dd76072214f62"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a089e727d5e46b9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34278,7 +34278,7 @@
         <x:v>MODMA / CHBMP</x:v>
       </x:c>
       <x:c r="D9" s="257" t="str">
-        <x:v>MODMA ID 13/14/17 已获批但官网当前不可达；CHBMP 已获批，首批 32/250 raw sessions 下载并完成 EDF 头审计。</x:v>
+        <x:v>MODMA ID 13/14/17 已获批，入口双端复测恢复并需重新登录；CHBMP 已获批，首批 32/250 raw sessions 下载并完成 EDF 头审计。</x:v>
       </x:c>
       <x:c r="E9" s="257" t="str">
         <x:v>MODMA 个人授权；CHBMP LORIS</x:v>
@@ -34370,7 +34370,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76b0eaeb1acf4c0c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46835b0972094a99"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update acquisition audit and direct-download workflow
</commit_message>
<xml_diff>
--- a/EEG_healthcare_disease_catalog_20260823.xlsx
+++ b/EEG_healthcare_disease_catalog_20260823.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R3fd9d4fe936b4764"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最终唯一下载清单" sheetId="2" r:id="R59a635ffaf1a4ba5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="修订记录" sheetId="8" r:id="Rb4dcd415287a4db9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R4b498e8ba22d40c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最终唯一下载清单" sheetId="2" r:id="Re03c1c9752344e32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="修订记录" sheetId="8" r:id="Rf668680bf5fb43c5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1426,6 +1426,12 @@
     <x:xf numFmtId="0" fontId="8" fillId="24" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="19" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="19" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="12" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="12" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
@@ -1488,12 +1494,6 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="11" fillId="21" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="19" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="19" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="10" fillId="20" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
@@ -1843,7 +1843,7 @@
         <x:v>服务器完成目录</x:v>
       </x:c>
       <x:c r="B7" s="247" t="str">
-        <x:v>74 units（含 TUH 重叠与非 raw 排除项）</x:v>
+        <x:v>80 units（含 TUH 重叠与非 raw 排除项）</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
@@ -1851,7 +1851,7 @@
         <x:v>独立 raw 已获取</x:v>
       </x:c>
       <x:c r="B8" s="247" t="str">
-        <x:v>67 units（疾病 55 / Health 12）</x:v>
+        <x:v>73 units（疾病 59 / Health 14）</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="34" customHeight="1">
@@ -1875,7 +1875,7 @@
         <x:v>下载执行队列</x:v>
       </x:c>
       <x:c r="B11" s="247" t="str">
-        <x:v>68 个仍可推进；4 个舍弃但保留目录证据</x:v>
+        <x:v>62 个仍可推进；4 个舍弃但保留目录证据</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="58" customHeight="1">
@@ -1891,7 +1891,7 @@
         <x:v>直接推进</x:v>
       </x:c>
       <x:c r="B13" s="213" t="str">
-        <x:v>19 个可直接下载；3 个只需登录；5 个需人工确认文件入口</x:v>
+        <x:v>2 个下载中；11 个可直接下载；3 个只需登录；5 个需人工确认文件入口</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="58" customHeight="1">
@@ -1899,7 +1899,7 @@
         <x:v>疾病/健康重点范围</x:v>
       </x:c>
       <x:c r="B14" s="213" t="str">
-        <x:v>146 units（疾病 109 / 健康 37）</x:v>
+        <x:v>146 units（疾病 108 / 健康 38）</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="58" customHeight="1">
@@ -1947,7 +1947,7 @@
         <x:v>口径提醒</x:v>
       </x:c>
       <x:c r="B20" s="215" t="str">
-        <x:v>67 是服务器目录与独立 raw 获取口径；57 / 43,627.8 h 是已有时长审计口径；346,490.7 h 是来源覆盖估计，三者不可混写。</x:v>
+        <x:v>73 是服务器目录与独立 raw 获取口径；57 / 43627.8 h 是已有时长审计口径；346490.7 h 是来源覆盖下界估计，三者不可混写。</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -1979,7 +1979,7 @@
         <x:v>分类逻辑</x:v>
       </x:c>
       <x:c r="B24" s="215" t="str">
-        <x:v>临床 MDD 属疾病；一般情绪/算术实验不是疾病。睡眠分期保留任务目录，同时按临床患者或健康队列进入疾病/健康重点范围。</x:v>
+        <x:v>临床 MDD 属疾病；一般情绪/算术实验不是疾病。DOD-H 为健康志愿者睡眠数据，归 Health；睡眠任务仍按患者/健康队列进入疾病/健康重点范围。</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -6223,7 +6223,7 @@
         <x:v>03_Consciousness_and_State/Sleep_Staging/DREAMER</x:v>
       </x:c>
       <x:c r="R71" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号 分类复核：DREAMER is an affective EEG/ECG experiment, not a sleep-health dataset. 分类复核：DREAMER is an affective EEG/ECG experiment, not a sleep-health dataset.</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 分类复核：DREAMER is an affective EEG/ECG experiment, not a sleep-health dataset. 分类复核：DREAMER is an affective EEG/ECG experiment, not a sleep-health dataset. 分类复核：DREAMER is an affective EEG/ECG experiment, not a sleep-health dataset. 分类复核：DREAMER is an affective EEG/ECG experiment, not a sleep-health dataset.</x:v>
       </x:c>
       <x:c r="S71" s="257"/>
       <x:c r="T71" s="257"/>
@@ -6234,10 +6234,10 @@
         <x:v>EEG-0122</x:v>
       </x:c>
       <x:c r="B72" s="275" t="str">
-        <x:v>03_Consciousness_and_State</x:v>
+        <x:v>08_Health_and_Population</x:v>
       </x:c>
       <x:c r="C72" s="275" t="str">
-        <x:v>Sleep_Staging</x:v>
+        <x:v>Sleep_Health_and_PSG</x:v>
       </x:c>
       <x:c r="D72" s="275" t="str">
         <x:v>Dreem Open Dataset – Healthy (DOD-H)</x:v>
@@ -6279,7 +6279,7 @@
         <x:v>Guillot et al. 2020</x:v>
       </x:c>
       <x:c r="Q72" s="275" t="str">
-        <x:v>03_Consciousness_and_State/Sleep_Staging/Dreem_Open_Datasets_DOD-H</x:v>
+        <x:v>08_Health_and_Population/Sleep_Health_and_PSG/Dreem_Open_Dataset_Healthy_DOD-H</x:v>
       </x:c>
       <x:c r="R72" s="275" t="str">
         <x:v>Dreem 官方仓库现指向 Zenodo:15900394；DOD-H 为 dodh.zip（21.9 GB）。旧 S3 桶已不存在，已更正入口。</x:v>
@@ -6407,10 +6407,10 @@
         <x:v>EEG-0125</x:v>
       </x:c>
       <x:c r="B75" s="257" t="str">
-        <x:v>03_Consciousness_and_State</x:v>
+        <x:v>02_Healthcare_and_Disease</x:v>
       </x:c>
       <x:c r="C75" s="257" t="str">
-        <x:v>Sleep_Staging</x:v>
+        <x:v>Clinical_Sleep_Disorders</x:v>
       </x:c>
       <x:c r="D75" s="257" t="str">
         <x:v>HMC (Haaglanden)</x:v>
@@ -6450,10 +6450,10 @@
         <x:v>Inter-database validation of a deep learning approach for automatic sleep scoring (Haaglanden Medisch Centrum sleep staging database). Alvarez-Estevez &amp; Rijsman, 2021, PLoS ONE 16(8):e0256111.</x:v>
       </x:c>
       <x:c r="Q75" s="257" t="str">
-        <x:v>03_Consciousness_and_State/Sleep_Staging/HMC_Haaglanden</x:v>
+        <x:v>02_Healthcare_and_Disease/Clinical_Sleep_Disorders/HMC_Haaglanden</x:v>
       </x:c>
       <x:c r="R75" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 分类复核：HMC is a clinical sleep-center cohort and belongs in the disease/clinical queue.</x:v>
       </x:c>
       <x:c r="S75" s="257"/>
       <x:c r="T75" s="257"/>
@@ -6569,7 +6569,7 @@
         <x:v>03_Consciousness_and_State/Sleep_Staging/MAHNOB-HCI</x:v>
       </x:c>
       <x:c r="R77" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号；2026-08-04去重：EEG-0184并入EEG-0129（MAHNOB-HCI official database identity） 分类复核：MAHNOB-HCI is multimodal affect recognition, not sleep staging. 分类复核：MAHNOB-HCI is multimodal affect recognition, not sleep staging.</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号；2026-08-04去重：EEG-0184并入EEG-0129（MAHNOB-HCI official database identity） 分类复核：MAHNOB-HCI is multimodal affect recognition, not sleep staging. 分类复核：MAHNOB-HCI is multimodal affect recognition, not sleep staging. 分类复核：MAHNOB-HCI is multimodal affect recognition, not sleep staging. 分类复核：MAHNOB-HCI is multimodal affect recognition, not sleep staging.</x:v>
       </x:c>
       <x:c r="S77" s="257"/>
       <x:c r="T77" s="257"/>
@@ -6977,7 +6977,7 @@
         <x:v>03_Consciousness_and_State/Sleep_Staging/Test-Retest_RestCog</x:v>
       </x:c>
       <x:c r="R84" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号 分类复核：RestCog is a healthy rest/cognitive-state benchmark, not a disease or population-health cohort. 分类复核：RestCog is a healthy rest/cognitive-state benchmark, not a disease or population-health cohort.</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 分类复核：RestCog is a healthy rest/cognitive-state benchmark, not a disease or population-health cohort. 分类复核：RestCog is a healthy rest/cognitive-state benchmark, not a disease or population-health cohort. 分类复核：RestCog is a healthy rest/cognitive-state benchmark, not a disease or population-health cohort. 分类复核：RestCog is a healthy rest/cognitive-state benchmark, not a disease or population-health cohort.</x:v>
       </x:c>
       <x:c r="S84" s="275"/>
       <x:c r="T84" s="275"/>
@@ -33274,7 +33274,7 @@
         <x:v>03_Consciousness_and_State/Sleep_Staging/ASCERTAIN</x:v>
       </x:c>
       <x:c r="R548" s="280" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号 分类复核：ASCERTAIN is an affect/personality experiment, not a sleep or clinical cohort. 分类复核：ASCERTAIN is an affect/personality experiment, not a sleep or clinical cohort.</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 分类复核：ASCERTAIN is an affect/personality experiment, not a sleep or clinical cohort. 分类复核：ASCERTAIN is an affect/personality experiment, not a sleep or clinical cohort. 分类复核：ASCERTAIN is an affect/personality experiment, not a sleep or clinical cohort. 分类复核：ASCERTAIN is an affect/personality experiment, not a sleep or clinical cohort.</x:v>
       </x:c>
       <x:c r="S548" s="280"/>
       <x:c r="T548" s="280"/>
@@ -34090,7 +34090,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a089e727d5e46b9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R334d792b93114e18"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34218,7 +34218,7 @@
         <x:v>疾病/健康 146 项</x:v>
       </x:c>
       <x:c r="D6" s="400" t="str">
-        <x:v>确认服务器完成 74 项、独立 raw 67 项、精确时长 57 项。</x:v>
+        <x:v>确认服务器完成 80 项、独立 raw 73 项、精确时长 57 项。</x:v>
       </x:c>
       <x:c r="E6" s="400" t="str">
         <x:v>SeaWulf VPN 只读快照</x:v>
@@ -34258,13 +34258,13 @@
         <x:v>EEG-0093 / EEG-0122</x:v>
       </x:c>
       <x:c r="D8" s="400" t="str">
-        <x:v>PD-Mortality 更新为 OpenNeuro ds007020 公开下载；DOD-H 更新为官方 Zenodo:15900394。</x:v>
+        <x:v>PD-Mortality 更新为 OpenNeuro ds007020；DOD-H 更新为官方 Zenodo:15900394，并按健康志愿者队列改归 Health。</x:v>
       </x:c>
       <x:c r="E8" s="400" t="str">
         <x:v>OpenNeuro ds007020；DOI:10.5281/zenodo.15900394</x:v>
       </x:c>
       <x:c r="F8" s="401" t="str">
-        <x:v>转为直接下载</x:v>
+        <x:v>两项已下载</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="54" customHeight="1">
@@ -34298,13 +34298,13 @@
         <x:v>19 public units</x:v>
       </x:c>
       <x:c r="D10" s="328" t="str">
-        <x:v>19 个直下单元总量超过当前 2.8 TB 空闲；先启动 EEG-Bench 4 项、PD-Mortality、DOD-H、HMC、UCDDB。</x:v>
+        <x:v>优先疾病/Health：Albrecht2019、Gruendler2009、Singh2020、Singh2021、PD-Mortality、DOD-H 已完成；HMC、UCDDB 下载中；其余 11 项暂不启动以保留预处理空间。</x:v>
       </x:c>
       <x:c r="E10" s="328" t="str">
-        <x:v>官方对象大小与服务器 df 审计</x:v>
+        <x:v>服务器 .download_complete 标记与 Slurm 2133731</x:v>
       </x:c>
       <x:c r="F10" s="329" t="str">
-        <x:v>Slurm 2133731</x:v>
+        <x:v>6 完成 / 2 下载中</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -34335,7 +34335,7 @@
         <x:v>QUEUE</x:v>
       </x:c>
       <x:c r="C12" s="328" t="str">
-        <x:v>68 actionable</x:v>
+        <x:v>62 actionable</x:v>
       </x:c>
       <x:c r="D12" s="328" t="str">
         <x:v>正式需申请 41 项：已申请 19 项，尚需申请 22 项；另有 4 项舍弃。</x:v>
@@ -34370,7 +34370,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46835b0972094a99"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8b134f152fa43e5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Surface verified EEG durations and fix MODMA launcher
</commit_message>
<xml_diff>
--- a/EEG_healthcare_disease_catalog_20260823.xlsx
+++ b/EEG_healthcare_disease_catalog_20260823.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R4b498e8ba22d40c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最终唯一下载清单" sheetId="2" r:id="Re03c1c9752344e32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="修订记录" sheetId="8" r:id="Rf668680bf5fb43c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rff0e6504b7d8439b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最终唯一下载清单" sheetId="2" r:id="R50a5f7171deb436a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="修订记录" sheetId="8" r:id="Rc55da9cd335f41ce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1580,7 +1580,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="RevisionLog20260823" displayName="RevisionLog20260823" ref="A1:F13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="RevisionLog20260823" displayName="RevisionLog20260823" ref="A1:F14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Change type"/>
@@ -1987,7 +1987,7 @@
         <x:v>受试者口径</x:v>
       </x:c>
       <x:c r="B25" s="215" t="str">
-        <x:v>99,515 dataset-subject entries（来源行合计；不是跨数据集去重后的唯一人数）</x:v>
+        <x:v>99,537 dataset-subject entries（来源行合计；不是跨数据集去重后的唯一人数）</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -2173,7 +2173,7 @@
         <x:v>02_Healthcare_and_Disease/Critical_Care_and_Coma/I-CARE</x:v>
       </x:c>
       <x:c r="R2" s="272" t="str">
-        <x:v>分类修正：心脏骤停后昏迷 ICU 连续 EEG 属临床疾病/重症监护；56,676 h 为完整 consortium 连续 EEG 文献口径，不等于本地已下载文件审计时长。</x:v>
+        <x:v>分类修正：心脏骤停后昏迷 ICU 连续 EEG 属临床疾病/重症监护；56,676 h 为完整 consortium 连续 EEG 文献口径，不等于本地已下载文件审计时长。 时长口径：56,676 h（论文/官网记录；I-CARE consortium paper; complete continuous EEG corpus）</x:v>
       </x:c>
       <x:c r="S2" s="272"/>
       <x:c r="T2" s="272" t="n">
@@ -2236,7 +2236,7 @@
         <x:v>08_Health_and_Population/Developmental_Clinical_Cohort/HBN_EEG_R1_ds005505</x:v>
       </x:c>
       <x:c r="R3" s="257" t="str">
-        <x:v>按 OpenNeuro 独立 release 去重；136 subjects、1,342 recordings、117.5 h。HBN 是广泛发育/精神健康表型队列，不等同于单一确诊疾病队列。</x:v>
+        <x:v>按 OpenNeuro 独立 release 去重；136 subjects、1,342 recordings、117.5 h。HBN 是广泛发育/精神健康表型队列，不等同于单一确诊疾病队列。 时长口径：117.5 h（论文/官网记录；EEGDash/OpenNeuro release metadata）</x:v>
       </x:c>
       <x:c r="S3" s="257"/>
       <x:c r="T3" s="257" t="n">
@@ -2299,7 +2299,7 @@
         <x:v>02_Healthcare_and_Disease/Mental_and_Developmental_Disorders/Albrecht2019</x:v>
       </x:c>
       <x:c r="R4" s="278" t="str">
-        <x:v>新增；EEG-Bench 论文与公开仓库交叉核验；51 h 为论文基准表记录</x:v>
+        <x:v>新增；EEG-Bench 论文与公开仓库交叉核验；51 h 为论文基准表记录 时长口径：51 h（论文/官网记录；EEG-Bench Table 1）</x:v>
       </x:c>
       <x:c r="S4" s="278"/>
       <x:c r="T4" s="278" t="n">
@@ -2362,7 +2362,7 @@
         <x:v>08_Health_and_Population/Mental_Health_Risk_Phenotype/Gruendler2009</x:v>
       </x:c>
       <x:c r="R5" s="278" t="str">
-        <x:v>新增；不标为确诊 OCD 疾病队列；22 h 为 EEG-Bench 表记录</x:v>
+        <x:v>新增；不标为确诊 OCD 疾病队列；22 h 为 EEG-Bench 表记录 时长口径：22 h（论文/官网记录；EEG-Bench Table 1）</x:v>
       </x:c>
       <x:c r="S5" s="278"/>
       <x:c r="T5" s="278" t="n">
@@ -2425,7 +2425,7 @@
         <x:v>02_Healthcare_and_Disease/Neurological_Disorders/Singh2020</x:v>
       </x:c>
       <x:c r="R6" s="278" t="str">
-        <x:v>新增；39 名与 7 h 由仓库/EEG-Bench 交叉核验</x:v>
+        <x:v>新增；39 名与 7 h 由仓库/EEG-Bench 交叉核验 时长口径：7 h（论文/官网记录；EEG-Bench Table 1）</x:v>
       </x:c>
       <x:c r="S6" s="278"/>
       <x:c r="T6" s="278" t="n">
@@ -2488,7 +2488,7 @@
         <x:v>02_Healthcare_and_Disease/Neurological_Disorders/Singh2021</x:v>
       </x:c>
       <x:c r="R7" s="278" t="str">
-        <x:v>新增；受试者与记录数分开；58 h 为 EEG-Bench 表记录</x:v>
+        <x:v>新增；受试者与记录数分开；58 h 为 EEG-Bench 表记录 时长口径：58 h（论文/官网记录；EEG-Bench Table 1）</x:v>
       </x:c>
       <x:c r="S7" s="278"/>
       <x:c r="T7" s="278" t="n">
@@ -2551,7 +2551,7 @@
         <x:v>08_Health_and_Population/Developmental_Clinical_Cohort/HBN_EEG_R2_ds005506</x:v>
       </x:c>
       <x:c r="R8" s="278" t="str">
-        <x:v>150 subjects、1,405 recordings、127.5 h；按 OpenNeuro 独立 release 去重。</x:v>
+        <x:v>150 subjects、1,405 recordings、127.5 h；按 OpenNeuro 独立 release 去重。 时长口径：127.5 h（论文/官网记录；EEGDash/OpenNeuro release metadata）</x:v>
       </x:c>
       <x:c r="S8" s="278"/>
       <x:c r="T8" s="278" t="n">
@@ -2614,7 +2614,7 @@
         <x:v>08_Health_and_Population/Developmental_Clinical_Cohort/HBN_EEG_R3_ds005507</x:v>
       </x:c>
       <x:c r="R9" s="278" t="str">
-        <x:v>184 subjects、1,812 recordings、158.8 h；按 OpenNeuro 独立 release 去重。</x:v>
+        <x:v>184 subjects、1,812 recordings、158.8 h；按 OpenNeuro 独立 release 去重。 时长口径：158.8 h（论文/官网记录；EEGDash/OpenNeuro release metadata）</x:v>
       </x:c>
       <x:c r="S9" s="278"/>
       <x:c r="T9" s="278" t="n">
@@ -2677,7 +2677,7 @@
         <x:v>08_Health_and_Population/Developmental_Clinical_Cohort/HBN_EEG_R4_ds005508</x:v>
       </x:c>
       <x:c r="R10" s="278" t="str">
-        <x:v>324 subjects、3,342 recordings、261.8 h；按 OpenNeuro 独立 release 去重。</x:v>
+        <x:v>324 subjects、3,342 recordings、261.8 h；按 OpenNeuro 独立 release 去重。 时长口径：261.8 h（论文/官网记录；EEGDash/OpenNeuro release metadata）</x:v>
       </x:c>
       <x:c r="S10" s="278"/>
       <x:c r="T10" s="278" t="n">
@@ -2740,7 +2740,7 @@
         <x:v>08_Health_and_Population/Developmental_Clinical_Cohort/HBN_EEG_R5_ds005509</x:v>
       </x:c>
       <x:c r="R11" s="278" t="str">
-        <x:v>330 subjects、3,326 recordings、255.3 h；按 OpenNeuro 独立 release 去重。</x:v>
+        <x:v>330 subjects、3,326 recordings、255.3 h；按 OpenNeuro 独立 release 去重。 时长口径：255.3 h（论文/官网记录；EEGDash/OpenNeuro release metadata）</x:v>
       </x:c>
       <x:c r="S11" s="278"/>
       <x:c r="T11" s="278" t="n">
@@ -2803,7 +2803,7 @@
         <x:v>08_Health_and_Population/Developmental_Clinical_Cohort/HBN_EEG_R6_ds005510</x:v>
       </x:c>
       <x:c r="R12" s="278" t="str">
-        <x:v>135 subjects、1,227 recordings、103.5 h；按 OpenNeuro 独立 release 去重。</x:v>
+        <x:v>135 subjects、1,227 recordings、103.5 h；按 OpenNeuro 独立 release 去重。 时长口径：103.5 h（论文/官网记录；EEGDash/OpenNeuro release metadata）</x:v>
       </x:c>
       <x:c r="S12" s="278"/>
       <x:c r="T12" s="278" t="n">
@@ -2866,7 +2866,7 @@
         <x:v>08_Health_and_Population/Developmental_Clinical_Cohort/HBN_EEG_R8_ds005512</x:v>
       </x:c>
       <x:c r="R13" s="278" t="str">
-        <x:v>257 subjects、2,320 recordings、179.1 h；按 OpenNeuro 独立 release 去重。</x:v>
+        <x:v>257 subjects、2,320 recordings、179.1 h；按 OpenNeuro 独立 release 去重。 时长口径：179.1 h（论文/官网记录；EEGDash/OpenNeuro release metadata）</x:v>
       </x:c>
       <x:c r="S13" s="278"/>
       <x:c r="T13" s="278" t="n">
@@ -2929,7 +2929,7 @@
         <x:v>08_Health_and_Population/Developmental_Clinical_Cohort/HBN_EEG_R9_ds005514</x:v>
       </x:c>
       <x:c r="R14" s="278" t="str">
-        <x:v>295 subjects、2,885 recordings、210.8 h；按 OpenNeuro 独立 release 去重。</x:v>
+        <x:v>295 subjects、2,885 recordings、210.8 h；按 OpenNeuro 独立 release 去重。 时长口径：210.8 h（论文/官网记录；EEGDash/OpenNeuro release metadata）</x:v>
       </x:c>
       <x:c r="S14" s="278"/>
       <x:c r="T14" s="278" t="n">
@@ -3049,10 +3049,12 @@
         <x:v>02_Biometrics_and_Disease/Epilepsy_and_Abnormalities/A_dataset_of_neonatal_EEG_recordings_with_seizures_annotations</x:v>
       </x:c>
       <x:c r="R16" s="275" t="str">
-        <x:v>EEG-0005 is the newer release and canonical download unit; EEG-0029 retained only in duplicate evidence</x:v>
+        <x:v>EEG-0005 is the newer release and canonical download unit; EEG-0029 retained only in duplicate evidence 时长口径：111.896 h（文件审计·部分范围；ACTUAL_DOWNLOADED_SCOPE_PARTIAL）</x:v>
       </x:c>
       <x:c r="S16" s="275"/>
-      <x:c r="T16" s="275"/>
+      <x:c r="T16" s="275" t="n">
+        <x:v>402825</x:v>
+      </x:c>
       <x:c r="U16" s="276"/>
     </x:row>
     <x:row r="17" ht="60" customHeight="1">
@@ -3106,10 +3108,12 @@
         <x:v>02_Biometrics_and_Disease/Epilepsy_and_Abnormalities/CHB-MIT</x:v>
       </x:c>
       <x:c r="R17" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：982.935 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S17" s="257"/>
-      <x:c r="T17" s="257"/>
+      <x:c r="T17" s="257" t="n">
+        <x:v>3538567</x:v>
+      </x:c>
       <x:c r="U17" s="213"/>
     </x:row>
     <x:row r="18" ht="60" customHeight="1">
@@ -3163,10 +3167,12 @@
         <x:v>02_Biometrics_and_Disease/Epilepsy_and_Abnormalities/Criteria_for_defining_interictal_epileptiform_discharges_in_EEG_a_clinical_validation_stud</x:v>
       </x:c>
       <x:c r="R18" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：0.351 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S18" s="275"/>
-      <x:c r="T18" s="275"/>
+      <x:c r="T18" s="275" t="n">
+        <x:v>1263</x:v>
+      </x:c>
       <x:c r="U18" s="276"/>
     </x:row>
     <x:row r="19" ht="60" customHeight="1">
@@ -3220,10 +3226,12 @@
         <x:v>02_Biometrics_and_Disease/Epilepsy_and_Abnormalities/HFO_High-Frequency_Oscillations</x:v>
       </x:c>
       <x:c r="R19" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：89.007 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S19" s="257"/>
-      <x:c r="T19" s="257"/>
+      <x:c r="T19" s="257" t="n">
+        <x:v>320425</x:v>
+      </x:c>
       <x:c r="U19" s="213"/>
     </x:row>
     <x:row r="20" ht="60" customHeight="1">
@@ -3277,10 +3285,12 @@
         <x:v>02_Biometrics_and_Disease/Epilepsy_and_Abnormalities/Intracranial_entrainment_reveals_statistical_learning_across_levels_of_abstraction</x:v>
       </x:c>
       <x:c r="R20" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：1.226 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S20" s="275"/>
-      <x:c r="T20" s="275"/>
+      <x:c r="T20" s="275" t="n">
+        <x:v>4414.859375</x:v>
+      </x:c>
       <x:c r="U20" s="276"/>
     </x:row>
     <x:row r="21" ht="60" customHeight="1">
@@ -3334,10 +3344,12 @@
         <x:v>02_Biometrics_and_Disease/Epilepsy_and_Abnormalities/SeizeIT2</x:v>
       </x:c>
       <x:c r="R21" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：11,626.249 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S21" s="257"/>
-      <x:c r="T21" s="257"/>
+      <x:c r="T21" s="257" t="n">
+        <x:v>41854496</x:v>
+      </x:c>
       <x:c r="U21" s="213"/>
     </x:row>
     <x:row r="22" ht="60" customHeight="1">
@@ -3391,10 +3403,12 @@
         <x:v>02_Biometrics_and_Disease/Epilepsy_and_Abnormalities/Siena_Scalp_EEG</x:v>
       </x:c>
       <x:c r="R22" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：141.021 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S22" s="275"/>
-      <x:c r="T22" s="275"/>
+      <x:c r="T22" s="275" t="n">
+        <x:v>507673.99999999994</x:v>
+      </x:c>
       <x:c r="U22" s="276"/>
     </x:row>
     <x:row r="23" ht="60" customHeight="1">
@@ -3448,10 +3462,12 @@
         <x:v>02_Biometrics_and_Disease/Epilepsy_and_Abnormalities/TUEP_TUH_Epilepsy</x:v>
       </x:c>
       <x:c r="R23" s="257" t="str">
-        <x:v>官方数据存在，但需申请、签署协议或获得权限；TUEP v3.1.0; subset of TUEG; do not add subjects or duration to TUEG totals</x:v>
+        <x:v>官方数据存在，但需申请、签署协议或获得权限；TUEP v3.1.0; subset of TUEG; do not add subjects or duration to TUEG totals 时长口径：626.766 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S23" s="257"/>
-      <x:c r="T23" s="257"/>
+      <x:c r="T23" s="257" t="n">
+        <x:v>2256359</x:v>
+      </x:c>
       <x:c r="U23" s="213"/>
     </x:row>
     <x:row r="24" ht="60" customHeight="1">
@@ -3505,10 +3521,12 @@
         <x:v>02_Biometrics_and_Disease/Epilepsy_and_Abnormalities/TUEV_TUH_Events</x:v>
       </x:c>
       <x:c r="R24" s="275" t="str">
-        <x:v>官方数据存在，但需申请、签署协议或获得权限；TUEV v2.0.1; subset of TUEG; do not add subjects or duration to TUEG totals</x:v>
+        <x:v>官方数据存在，但需申请、签署协议或获得权限；TUEV v2.0.1; subset of TUEG; do not add subjects or duration to TUEG totals 时长口径：148.745 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S24" s="275"/>
-      <x:c r="T24" s="275"/>
+      <x:c r="T24" s="275" t="n">
+        <x:v>535481</x:v>
+      </x:c>
       <x:c r="U24" s="276"/>
     </x:row>
     <x:row r="25" ht="60" customHeight="1">
@@ -3562,10 +3580,12 @@
         <x:v>02_Biometrics_and_Disease/Epilepsy_and_Abnormalities/TUSL_TUH_Slowing</x:v>
       </x:c>
       <x:c r="R25" s="257" t="str">
-        <x:v>官方数据存在，但需申请、签署协议或获得权限；TUSL v2.0.1; subset of TUEG; do not add subjects or duration to TUEG totals</x:v>
+        <x:v>官方数据存在，但需申请、签署协议或获得权限；TUSL v2.0.1; subset of TUEG; do not add subjects or duration to TUEG totals 时长口径：27.596 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S25" s="257"/>
-      <x:c r="T25" s="257"/>
+      <x:c r="T25" s="257" t="n">
+        <x:v>99347</x:v>
+      </x:c>
       <x:c r="U25" s="213"/>
     </x:row>
     <x:row r="26" ht="60" customHeight="1">
@@ -3619,10 +3639,12 @@
         <x:v>02_Biometrics_and_Disease/Epilepsy_and_Abnormalities/TUSZ_TUH_Seizure</x:v>
       </x:c>
       <x:c r="R26" s="275" t="str">
-        <x:v>官方数据存在，但需申请、签署协议或获得权限；TUSZ v2.0.6; subset of TUEG; do not add subjects or duration to TUEG totals</x:v>
+        <x:v>官方数据存在，但需申请、签署协议或获得权限；TUSZ v2.0.6; subset of TUEG; do not add subjects or duration to TUEG totals 时长口径：1,474.787 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S26" s="275"/>
-      <x:c r="T26" s="275"/>
+      <x:c r="T26" s="275" t="n">
+        <x:v>5309234</x:v>
+      </x:c>
       <x:c r="U26" s="276"/>
     </x:row>
     <x:row r="27" ht="60" customHeight="1">
@@ -3676,10 +3698,12 @@
         <x:v>02_Biometrics_and_Disease/Neurodegenerative_Disorders/AD65_Alzheimer_FTD</x:v>
       </x:c>
       <x:c r="R27" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：39.006 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S27" s="257"/>
-      <x:c r="T27" s="257"/>
+      <x:c r="T27" s="257" t="n">
+        <x:v>140421.42000000022</x:v>
+      </x:c>
       <x:c r="U27" s="213"/>
     </x:row>
     <x:row r="28" ht="60" customHeight="1">
@@ -3733,10 +3757,12 @@
         <x:v>02_Biometrics_and_Disease/Neurodegenerative_Disorders/Alzheimer_Risk_Classification_Sample-enrichment_EEG</x:v>
       </x:c>
       <x:c r="R28" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：3.912 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S28" s="275"/>
-      <x:c r="T28" s="275"/>
+      <x:c r="T28" s="275" t="n">
+        <x:v>14081.599999999999</x:v>
+      </x:c>
       <x:c r="U28" s="276"/>
     </x:row>
     <x:row r="29" ht="60" customHeight="1">
@@ -3792,10 +3818,12 @@
         <x:v>02_Biometrics_and_Disease/Neurodegenerative_Disorders/EEG_p-adic_quantum_potential_accurately_identifies_depression_schizophrenia_and_cognitive_</x:v>
       </x:c>
       <x:c r="R29" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号；2026-08-04去重：EEG-0046并入EEG-0045（Project download-content audit: P-ADIC source duplication）</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号；2026-08-04去重：EEG-0046并入EEG-0045（Project download-content audit: P-ADIC source duplication） 时长口径：84.3 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S29" s="257"/>
-      <x:c r="T29" s="257"/>
+      <x:c r="T29" s="257" t="n">
+        <x:v>303479.05400000006</x:v>
+      </x:c>
       <x:c r="U29" s="213"/>
     </x:row>
     <x:row r="30" ht="60" customHeight="1">
@@ -3849,10 +3877,12 @@
         <x:v>02_Biometrics_and_Disease/Neurodegenerative_Disorders/Resting-state_high-density_EEG_using_EGI_GES_300_for_healthy_elders_SCD_MCI_and_Alzheimer_</x:v>
       </x:c>
       <x:c r="R30" s="275" t="str">
-        <x:v>官方数据存在，但需申请、签署协议或获得权限</x:v>
+        <x:v>官方数据存在，但需申请、签署协议或获得权限 时长口径：1.5 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S30" s="275"/>
-      <x:c r="T30" s="275"/>
+      <x:c r="T30" s="275" t="n">
+        <x:v>5400</x:v>
+      </x:c>
       <x:c r="U30" s="276"/>
     </x:row>
     <x:row r="31" ht="60" customHeight="1">
@@ -3906,10 +3936,12 @@
         <x:v>02_Biometrics_and_Disease/Mental_and_Developmental_Disorders/Depression_resting_BDI</x:v>
       </x:c>
       <x:c r="R31" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：23.36 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S31" s="257"/>
-      <x:c r="T31" s="257"/>
+      <x:c r="T31" s="257" t="n">
+        <x:v>84094.76800000005</x:v>
+      </x:c>
       <x:c r="U31" s="213"/>
     </x:row>
     <x:row r="32" ht="60" customHeight="1">
@@ -4022,10 +4054,12 @@
         <x:v>02_Biometrics_and_Disease/Mental_and_Developmental_Disorders/FEPCR</x:v>
       </x:c>
       <x:c r="R33" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：12.265 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S33" s="257"/>
-      <x:c r="T33" s="257"/>
+      <x:c r="T33" s="257" t="n">
+        <x:v>44154.998287400005</x:v>
+      </x:c>
       <x:c r="U33" s="213"/>
     </x:row>
     <x:row r="34" ht="60" customHeight="1">
@@ -4079,10 +4113,12 @@
         <x:v>02_Biometrics_and_Disease/Mental_and_Developmental_Disorders/Fribourg_Ultimatum_Game_in_Schizophrenia_Study</x:v>
       </x:c>
       <x:c r="R34" s="275" t="str">
-        <x:v>官方数据存在，但需申请、签署协议或获得权限</x:v>
+        <x:v>官方数据存在，但需申请、签署协议或获得权限 时长口径：12.057 h（文件审计·部分范围；ACTUAL_DOWNLOADED_SCOPE_PARTIAL）</x:v>
       </x:c>
       <x:c r="S34" s="275"/>
-      <x:c r="T34" s="275"/>
+      <x:c r="T34" s="275" t="n">
+        <x:v>43404</x:v>
+      </x:c>
       <x:c r="U34" s="276"/>
     </x:row>
     <x:row r="35" ht="60" customHeight="1">
@@ -4140,10 +4176,12 @@
         <x:v>02_Biometrics_and_Disease/Mental_and_Developmental_Disorders/MDD_Mumtaz</x:v>
       </x:c>
       <x:c r="R35" s="257" t="str">
-        <x:v>官方数据存在，但需申请、签署协议或获得权限</x:v>
+        <x:v>官方数据存在，但需申请、签署协议或获得权限 时长口径：20.556 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S35" s="257"/>
-      <x:c r="T35" s="257"/>
+      <x:c r="T35" s="257" t="n">
+        <x:v>74001</x:v>
+      </x:c>
       <x:c r="U35" s="213"/>
     </x:row>
     <x:row r="36" ht="60" customHeight="1">
@@ -4197,10 +4235,12 @@
         <x:v>02_Biometrics_and_Disease/Mental_and_Developmental_Disorders/Power_Spectral_Density-Based_Resting-State_EEG_Classification_of_First-Episode_Psychosis</x:v>
       </x:c>
       <x:c r="R36" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：6.05 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S36" s="275"/>
-      <x:c r="T36" s="275"/>
+      <x:c r="T36" s="275" t="n">
+        <x:v>21780</x:v>
+      </x:c>
       <x:c r="U36" s="276"/>
     </x:row>
     <x:row r="37" ht="60" customHeight="1">
@@ -4254,10 +4294,12 @@
         <x:v>02_Biometrics_and_Disease/Neurological_Disorders/Acute_Mild_TBI_DPX_Cognitive-control_EEG</x:v>
       </x:c>
       <x:c r="R37" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：124.273 h（文件审计·部分范围；ACTUAL_DOWNLOADED_SCOPE_PARTIAL）</x:v>
       </x:c>
       <x:c r="S37" s="257"/>
-      <x:c r="T37" s="257"/>
+      <x:c r="T37" s="257" t="n">
+        <x:v>447381.55</x:v>
+      </x:c>
       <x:c r="U37" s="213"/>
     </x:row>
     <x:row r="38" ht="60" customHeight="1">
@@ -4313,10 +4355,12 @@
         <x:v>02_Biometrics_and_Disease/Neurological_Disorders/Acute_Stroke_Motor_Imagery_EEG_Dataset</x:v>
       </x:c>
       <x:c r="R38" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：2.667 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S38" s="275"/>
-      <x:c r="T38" s="275"/>
+      <x:c r="T38" s="275" t="n">
+        <x:v>9600</x:v>
+      </x:c>
       <x:c r="U38" s="276"/>
     </x:row>
     <x:row r="39" ht="60" customHeight="1">
@@ -4370,10 +4414,12 @@
         <x:v>02_Biometrics_and_Disease/Neurological_Disorders/ALS-Spelling_EEG-ET</x:v>
       </x:c>
       <x:c r="R39" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：66.323 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S39" s="257"/>
-      <x:c r="T39" s="257"/>
+      <x:c r="T39" s="257" t="n">
+        <x:v>238763</x:v>
+      </x:c>
       <x:c r="U39" s="213"/>
     </x:row>
     <x:row r="40" ht="60" customHeight="1">
@@ -4666,10 +4712,12 @@
         <x:v>02_Biometrics_and_Disease/Neurological_Disorders/BNCI_008-2014_P300_speller_ALS</x:v>
       </x:c>
       <x:c r="R44" s="275" t="str">
-        <x:v>官方数据存在，但需申请、签署协议或获得权限；2026-08-04去重：EEG-0072并入EEG-0071（BNCI 008-2014 / MOABB BNCI2014_008）</x:v>
+        <x:v>官方数据存在，但需申请、签署协议或获得权限；2026-08-04去重：EEG-0072并入EEG-0071（BNCI 008-2014 / MOABB BNCI2014_008） 时长口径：3.018 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S44" s="275"/>
-      <x:c r="T44" s="275"/>
+      <x:c r="T44" s="275" t="n">
+        <x:v>10865.75</x:v>
+      </x:c>
       <x:c r="U44" s="276"/>
     </x:row>
     <x:row r="45" ht="60" customHeight="1">
@@ -4723,10 +4771,12 @@
         <x:v>02_Biometrics_and_Disease/Neurological_Disorders/CCEP_ECoG_Dataset_across_age_4-51</x:v>
       </x:c>
       <x:c r="R45" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：89.391 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S45" s="257"/>
-      <x:c r="T45" s="257"/>
+      <x:c r="T45" s="257" t="n">
+        <x:v>321807.6762644932</x:v>
+      </x:c>
       <x:c r="U45" s="213"/>
     </x:row>
     <x:row r="46" ht="60" customHeight="1">
@@ -4780,10 +4830,12 @@
         <x:v>02_Biometrics_and_Disease/Neurological_Disorders/Dataset_of_electrophysiological_signals_EEG_ECG_EMG_during_Music_therapy_with_adult_burn_p</x:v>
       </x:c>
       <x:c r="R46" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：10.941 h（文件审计·部分范围；ACTUAL_DOWNLOADED_SCOPE_PARTIAL）</x:v>
       </x:c>
       <x:c r="S46" s="275"/>
-      <x:c r="T46" s="275"/>
+      <x:c r="T46" s="275" t="n">
+        <x:v>39386</x:v>
+      </x:c>
       <x:c r="U46" s="276"/>
     </x:row>
     <x:row r="47" ht="60" customHeight="1">
@@ -4955,10 +5007,12 @@
         <x:v>02_Biometrics_and_Disease/Neurological_Disorders/EEG_3-Stim_Auditory_Oddball_and_Rest_in_Parkinson_s</x:v>
       </x:c>
       <x:c r="R49" s="257" t="str">
-        <x:v>官方数据存在，但需申请、签署协议或获得权限</x:v>
+        <x:v>官方数据存在，但需申请、签署协议或获得权限 时长口径：12.76 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S49" s="257"/>
-      <x:c r="T49" s="257"/>
+      <x:c r="T49" s="257" t="n">
+        <x:v>45935.70000000001</x:v>
+      </x:c>
       <x:c r="U49" s="213"/>
     </x:row>
     <x:row r="50" ht="60" customHeight="1">
@@ -5012,10 +5066,12 @@
         <x:v>02_Biometrics_and_Disease/Neurological_Disorders/EEG_Reinforcement_Learning_in_Parkinson_s</x:v>
       </x:c>
       <x:c r="R50" s="275" t="str">
-        <x:v>官方数据存在，但需申请、签署协议或获得权限</x:v>
+        <x:v>官方数据存在，但需申请、签署协议或获得权限 时长口径：35.381 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S50" s="275"/>
-      <x:c r="T50" s="275"/>
+      <x:c r="T50" s="275" t="n">
+        <x:v>127372.59999999993</x:v>
+      </x:c>
       <x:c r="U50" s="276"/>
     </x:row>
     <x:row r="51" ht="60" customHeight="1">
@@ -5069,10 +5125,12 @@
         <x:v>02_Biometrics_and_Disease/Neurological_Disorders/EEG_Simon_Conflict_in_Parkinson_s</x:v>
       </x:c>
       <x:c r="R51" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：48.535 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S51" s="257"/>
-      <x:c r="T51" s="257"/>
+      <x:c r="T51" s="257" t="n">
+        <x:v>174725.50000000006</x:v>
+      </x:c>
       <x:c r="U51" s="213"/>
     </x:row>
     <x:row r="52" ht="60" customHeight="1">
@@ -5126,10 +5184,12 @@
         <x:v>02_Biometrics_and_Disease/Neurological_Disorders/EEG_Three-Stim_Auditory_Oddball_and_Rest_in_Acute_and_Chronic_TBI</x:v>
       </x:c>
       <x:c r="R52" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：140.8 h（文件审计·部分范围；ACTUAL_DOWNLOADED_SCOPE_PARTIAL）</x:v>
       </x:c>
       <x:c r="S52" s="275"/>
-      <x:c r="T52" s="275"/>
+      <x:c r="T52" s="275" t="n">
+        <x:v>506878.3499999997</x:v>
+      </x:c>
       <x:c r="U52" s="276"/>
     </x:row>
     <x:row r="53" ht="60" customHeight="1">
@@ -5183,10 +5243,12 @@
         <x:v>02_Biometrics_and_Disease/Neurological_Disorders/Human_Spinal-cord_Somatosensory_Evoked_Potentials_EEG</x:v>
       </x:c>
       <x:c r="R53" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：43.49 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S53" s="257"/>
-      <x:c r="T53" s="257"/>
+      <x:c r="T53" s="257" t="n">
+        <x:v>156563.65440000014</x:v>
+      </x:c>
       <x:c r="U53" s="213"/>
     </x:row>
     <x:row r="54" ht="60" customHeight="1">
@@ -5240,10 +5302,12 @@
         <x:v>02_Biometrics_and_Disease/Neurological_Disorders/Intraoperative_Medianus-tibialis_Stimulation_EEG</x:v>
       </x:c>
       <x:c r="R54" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：11.763 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S54" s="275"/>
-      <x:c r="T54" s="275"/>
+      <x:c r="T54" s="275" t="n">
+        <x:v>42347</x:v>
+      </x:c>
       <x:c r="U54" s="276"/>
     </x:row>
     <x:row r="55" ht="60" customHeight="1">
@@ -5301,10 +5365,12 @@
         <x:v>02_Biometrics_and_Disease/Neurological_Disorders/Liu2024</x:v>
       </x:c>
       <x:c r="R55" s="257" t="str">
-        <x:v>官方数据存在，但需申请、签署协议或获得权限</x:v>
+        <x:v>官方数据存在，但需申请、签署协议或获得权限 时长口径：4.444 h（文件审计·部分范围；ACTUAL_DOWNLOADED_SCOPE_PARTIAL）</x:v>
       </x:c>
       <x:c r="S55" s="257"/>
-      <x:c r="T55" s="257"/>
+      <x:c r="T55" s="257" t="n">
+        <x:v>16000</x:v>
+      </x:c>
       <x:c r="U55" s="213"/>
     </x:row>
     <x:row r="56" ht="60" customHeight="1">
@@ -5360,10 +5426,12 @@
         <x:v>02_Biometrics_and_Disease/Neurological_Disorders/Lower-Limb-MI_stroke</x:v>
       </x:c>
       <x:c r="R56" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号；2026-08-04去重：EEG-0396并入EEG-0085（Figshare article 27130299）</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号；2026-08-04去重：EEG-0396并入EEG-0085（Figshare article 27130299） 时长口径：33.448 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S56" s="275"/>
-      <x:c r="T56" s="275"/>
+      <x:c r="T56" s="275" t="n">
+        <x:v>120413</x:v>
+      </x:c>
       <x:c r="U56" s="276"/>
     </x:row>
     <x:row r="57" ht="60" customHeight="1">
@@ -5419,10 +5487,12 @@
         <x:v>02_Biometrics_and_Disease/Neurological_Disorders/Migrainedb</x:v>
       </x:c>
       <x:c r="R57" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：21.232 h（文件审计·部分范围；ACTUAL_DOWNLOADED_SCOPE_PARTIAL）</x:v>
       </x:c>
       <x:c r="S57" s="257"/>
-      <x:c r="T57" s="257"/>
+      <x:c r="T57" s="257" t="n">
+        <x:v>76436</x:v>
+      </x:c>
       <x:c r="U57" s="213"/>
     </x:row>
     <x:row r="58" ht="60" customHeight="1">
@@ -5476,10 +5546,12 @@
         <x:v>02_Biometrics_and_Disease/Neurological_Disorders/Mu_and_Beta_Oscillatory_Changes_during_a_motor_task_following_Rehabilitation_in_Chronic_MC</x:v>
       </x:c>
       <x:c r="R58" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：12.291 h（文件审计·部分范围；ACTUAL_DOWNLOADED_SCOPE_PARTIAL）</x:v>
       </x:c>
       <x:c r="S58" s="275"/>
-      <x:c r="T58" s="275"/>
+      <x:c r="T58" s="275" t="n">
+        <x:v>44247.16</x:v>
+      </x:c>
       <x:c r="U58" s="276"/>
     </x:row>
     <x:row r="59" ht="60" customHeight="1">
@@ -5590,10 +5662,12 @@
         <x:v>02_Biometrics_and_Disease/Neurological_Disorders/PD-EEG_Resting-State_Walking_EEG</x:v>
       </x:c>
       <x:c r="R60" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：19.489 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S60" s="275"/>
-      <x:c r="T60" s="275"/>
+      <x:c r="T60" s="275" t="n">
+        <x:v>70159.26000000001</x:v>
+      </x:c>
       <x:c r="U60" s="276"/>
     </x:row>
     <x:row r="61" ht="60" customHeight="1">
@@ -5704,10 +5778,12 @@
         <x:v>02_Biometrics_and_Disease/Neurological_Disorders/PD31_Parkinson</x:v>
       </x:c>
       <x:c r="R62" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：2.518 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S62" s="275"/>
-      <x:c r="T62" s="275"/>
+      <x:c r="T62" s="275" t="n">
+        <x:v>9064</x:v>
+      </x:c>
       <x:c r="U62" s="276"/>
     </x:row>
     <x:row r="63" ht="60" customHeight="1">
@@ -5993,10 +6069,12 @@
         <x:v>02_Biometrics_and_Disease/Clinical_Abnormalities/TUAB_TUH_Abnormal</x:v>
       </x:c>
       <x:c r="R67" s="257" t="str">
-        <x:v>官方数据存在，但需申请、签署协议或获得权限；TUAB v3.0.1; subset of TUEG; do not add subjects or duration to TUEG totals</x:v>
+        <x:v>官方数据存在，但需申请、签署协议或获得权限；TUAB v3.0.1; subset of TUEG; do not add subjects or duration to TUEG totals 时长口径：1,141.002 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S67" s="257"/>
-      <x:c r="T67" s="257"/>
+      <x:c r="T67" s="257" t="n">
+        <x:v>4107607.9999999995</x:v>
+      </x:c>
       <x:c r="U67" s="213"/>
     </x:row>
     <x:row r="68" ht="60" customHeight="1">
@@ -6223,7 +6301,7 @@
         <x:v>03_Consciousness_and_State/Sleep_Staging/DREAMER</x:v>
       </x:c>
       <x:c r="R71" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号 分类复核：DREAMER is an affective EEG/ECG experiment, not a sleep-health dataset. 分类复核：DREAMER is an affective EEG/ECG experiment, not a sleep-health dataset. 分类复核：DREAMER is an affective EEG/ECG experiment, not a sleep-health dataset. 分类复核：DREAMER is an affective EEG/ECG experiment, not a sleep-health dataset.</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 分类复核：DREAMER is an affective EEG/ECG experiment, not a sleep-health dataset. 分类复核：DREAMER is an affective EEG/ECG experiment, not a sleep-health dataset. 分类复核：DREAMER is an affective EEG/ECG experiment, not a sleep-health dataset. 分类复核：DREAMER is an affective EEG/ECG experiment, not a sleep-health dataset. 分类复核：DREAMER is an affective EEG/ECG experiment, not a sleep-health dataset.</x:v>
       </x:c>
       <x:c r="S71" s="257"/>
       <x:c r="T71" s="257"/>
@@ -6282,10 +6360,12 @@
         <x:v>08_Health_and_Population/Sleep_Health_and_PSG/Dreem_Open_Dataset_Healthy_DOD-H</x:v>
       </x:c>
       <x:c r="R72" s="275" t="str">
-        <x:v>Dreem 官方仓库现指向 Zenodo:15900394；DOD-H 为 dodh.zip（21.9 GB）。旧 S3 桶已不存在，已更正入口。</x:v>
+        <x:v>Dreem 官方仓库现指向 Zenodo:15900394；DOD-H 为 dodh.zip（21.9 GB）。旧 S3 桶已不存在，已更正入口。 时长口径：205.542 h（论文换算·明确范围；Common Sleep Data Pipeline Table 1: 24,665 retained 30-s epochs / 120 = 205.542 h; CSDP DOD-H subset (25 records; catalog release is wider)）</x:v>
       </x:c>
       <x:c r="S72" s="275"/>
-      <x:c r="T72" s="275"/>
+      <x:c r="T72" s="275" t="n">
+        <x:v>739950</x:v>
+      </x:c>
       <x:c r="U72" s="276"/>
     </x:row>
     <x:row r="73" ht="60" customHeight="1">
@@ -6453,7 +6533,7 @@
         <x:v>02_Healthcare_and_Disease/Clinical_Sleep_Disorders/HMC_Haaglanden</x:v>
       </x:c>
       <x:c r="R75" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号 分类复核：HMC is a clinical sleep-center cohort and belongs in the disease/clinical queue.</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 分类复核：HMC is a clinical sleep-center cohort and belongs in the disease/clinical queue. 分类复核：HMC is a clinical sleep-center cohort and belongs in the disease/clinical queue.</x:v>
       </x:c>
       <x:c r="S75" s="257"/>
       <x:c r="T75" s="257"/>
@@ -6569,7 +6649,7 @@
         <x:v>03_Consciousness_and_State/Sleep_Staging/MAHNOB-HCI</x:v>
       </x:c>
       <x:c r="R77" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号；2026-08-04去重：EEG-0184并入EEG-0129（MAHNOB-HCI official database identity） 分类复核：MAHNOB-HCI is multimodal affect recognition, not sleep staging. 分类复核：MAHNOB-HCI is multimodal affect recognition, not sleep staging. 分类复核：MAHNOB-HCI is multimodal affect recognition, not sleep staging. 分类复核：MAHNOB-HCI is multimodal affect recognition, not sleep staging.</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号；2026-08-04去重：EEG-0184并入EEG-0129（MAHNOB-HCI official database identity） 分类复核：MAHNOB-HCI is multimodal affect recognition, not sleep staging. 分类复核：MAHNOB-HCI is multimodal affect recognition, not sleep staging. 分类复核：MAHNOB-HCI is multimodal affect recognition, not sleep staging. 分类复核：MAHNOB-HCI is multimodal affect recognition, not sleep staging. 分类复核：MAHNOB-HCI is multimodal affect recognition, not sleep staging.</x:v>
       </x:c>
       <x:c r="S77" s="257"/>
       <x:c r="T77" s="257"/>
@@ -6803,10 +6883,12 @@
         <x:v>03_Consciousness_and_State/Sleep_Staging/PhysioNet_Challenge_2018_Sleep_Arousal_Database</x:v>
       </x:c>
       <x:c r="R81" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：7,061.217 h（论文换算·明确范围；Common Sleep Data Pipeline Table 1: 847,346 retained 30-s epochs / 120 = 7061.217 h; CSDP subset (919 records; catalog release is wider)）</x:v>
       </x:c>
       <x:c r="S81" s="257"/>
-      <x:c r="T81" s="257"/>
+      <x:c r="T81" s="257" t="n">
+        <x:v>25420380</x:v>
+      </x:c>
       <x:c r="U81" s="213"/>
     </x:row>
     <x:row r="82" ht="60" customHeight="1">
@@ -6917,10 +6999,12 @@
         <x:v>03_Consciousness_and_State/Sleep_Staging/Sleep-EDF_Expanded</x:v>
       </x:c>
       <x:c r="R83" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：3,575.592 h（论文换算·明确范围；Common Sleep Data Pipeline Table 1: 429,071 retained 30-s epochs / 120 = 3575.592 h; CSDP Sleep-EDF SC+ST analysed subset）</x:v>
       </x:c>
       <x:c r="S83" s="257"/>
-      <x:c r="T83" s="257"/>
+      <x:c r="T83" s="257" t="n">
+        <x:v>12872130</x:v>
+      </x:c>
       <x:c r="U83" s="213"/>
     </x:row>
     <x:row r="84" ht="60" customHeight="1">
@@ -6977,7 +7061,7 @@
         <x:v>03_Consciousness_and_State/Sleep_Staging/Test-Retest_RestCog</x:v>
       </x:c>
       <x:c r="R84" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号 分类复核：RestCog is a healthy rest/cognitive-state benchmark, not a disease or population-health cohort. 分类复核：RestCog is a healthy rest/cognitive-state benchmark, not a disease or population-health cohort. 分类复核：RestCog is a healthy rest/cognitive-state benchmark, not a disease or population-health cohort. 分类复核：RestCog is a healthy rest/cognitive-state benchmark, not a disease or population-health cohort.</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 分类复核：RestCog is a healthy rest/cognitive-state benchmark, not a disease or population-health cohort. 分类复核：RestCog is a healthy rest/cognitive-state benchmark, not a disease or population-health cohort. 分类复核：RestCog is a healthy rest/cognitive-state benchmark, not a disease or population-health cohort. 分类复核：RestCog is a healthy rest/cognitive-state benchmark, not a disease or population-health cohort. 分类复核：RestCog is a healthy rest/cognitive-state benchmark, not a disease or population-health cohort.</x:v>
       </x:c>
       <x:c r="S84" s="275"/>
       <x:c r="T84" s="275"/>
@@ -17347,10 +17431,12 @@
         <x:v>02_Biometrics_and_Disease/Development_and_Lifespan/Infant_First-year_Resting_EEG_Dataset</x:v>
       </x:c>
       <x:c r="R264" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：22.839 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S264" s="275"/>
-      <x:c r="T264" s="275"/>
+      <x:c r="T264" s="275" t="n">
+        <x:v>82220</x:v>
+      </x:c>
       <x:c r="U264" s="276"/>
     </x:row>
     <x:row r="265" ht="60" customHeight="1">
@@ -17404,10 +17490,12 @@
         <x:v>02_Biometrics_and_Disease/Development_and_Lifespan/SFARI_EEG_multi-paradigm_dataset</x:v>
       </x:c>
       <x:c r="R265" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：229.423 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S265" s="257"/>
-      <x:c r="T265" s="257"/>
+      <x:c r="T265" s="257" t="n">
+        <x:v>825921.681640625</x:v>
+      </x:c>
       <x:c r="U265" s="213"/>
     </x:row>
     <x:row r="266" ht="60" customHeight="1">
@@ -20010,10 +20098,12 @@
         <x:v>02_Biometrics_and_Disease/Clinical_Abnormalities/TUEG_TUH_EEG_Corpus</x:v>
       </x:c>
       <x:c r="R309" s="257" t="str">
-        <x:v>Restored as an independent download unit. Current official release: v2.0.2. User-provided v2.0.1 audit: 97,478,219 s = 27,077.3 h; EDF directory about 1,643 GB (du -sBG: 1,646G). All TUH subsets overlap TUEG and must not be added to its totals.</x:v>
+        <x:v>Restored as an independent download unit. Current official release: v2.0.2. User-provided v2.0.1 audit: 97,478,219 s = 27,077.3 h; EDF directory about 1,643 GB (du -sBG: 1,646G). All TUH subsets overlap TUEG and must not be added to its totals. 时长口径：27,077.3 h（发布/下载范围；未核验）</x:v>
       </x:c>
       <x:c r="S309" s="257"/>
-      <x:c r="T309" s="257"/>
+      <x:c r="T309" s="257" t="n">
+        <x:v>97478280</x:v>
+      </x:c>
       <x:c r="U309" s="213"/>
     </x:row>
     <x:row r="310" ht="60" customHeight="1">
@@ -20557,10 +20647,12 @@
         <x:v>02_Healthcare_and_Disease/Epilepsy_and_Seizure_Monitoring/SeizeIT1</x:v>
       </x:c>
       <x:c r="R318" s="278" t="str">
-        <x:v>NeuroAtlas Figure 2 labels 5.9k h; the current SzCORE public benchmark lists 4,211 h for 42 subjects. The hour field stays non-exact in the master row and both scopes are preserved in the comparison sheet.</x:v>
+        <x:v>NeuroAtlas Figure 2 labels 5.9k h; the current SzCORE public benchmark lists 4,211 h for 42 subjects. The hour field stays non-exact in the master row and both scopes are preserved in the comparison sheet. 时长口径：5,900 h（论文/官网记录；NeuroAtlas Figure 2; SzCORE lists 4,211 h for the current public benchmark scope）</x:v>
       </x:c>
       <x:c r="S318" s="278"/>
-      <x:c r="T318" s="278"/>
+      <x:c r="T318" s="278" t="n">
+        <x:v>21240000</x:v>
+      </x:c>
       <x:c r="U318" s="247"/>
     </x:row>
     <x:row r="319" ht="60" customHeight="1">
@@ -20616,10 +20708,12 @@
         <x:v>02_Healthcare_and_Disease/Clinical_Sleep_Disorders/DCSM</x:v>
       </x:c>
       <x:c r="R319" s="278" t="str">
-        <x:v>Official archive confirms 255 anonymized overnight clinical PSGs. No official total-hour figure was found, so duration is left blank.</x:v>
+        <x:v>Official archive confirms 255 anonymized overnight clinical PSGs. No official total-hour figure was found, so duration is left blank. 时长口径：4,824.492 h（论文换算·明确范围；Common Sleep Data Pipeline Table 1: 578,939 retained 30-s epochs / 120 = 4824.492 h; CSDP analysed cohort）</x:v>
       </x:c>
       <x:c r="S319" s="278"/>
-      <x:c r="T319" s="278"/>
+      <x:c r="T319" s="278" t="n">
+        <x:v>17368170</x:v>
+      </x:c>
       <x:c r="U319" s="247" t="n">
         <x:v>255</x:v>
       </x:c>
@@ -20799,10 +20893,12 @@
         <x:v>02_Healthcare_and_Disease/Sleep_Disordered_Breathing/UCDDB</x:v>
       </x:c>
       <x:c r="R322" s="278" t="str">
-        <x:v>Official PhysioNet page confirms 25 subjects and 25 full overnight PSGs. Total hours are not inferred from file size or an assumed night length.</x:v>
+        <x:v>Official PhysioNet page confirms 25 subjects and 25 full overnight PSGs. Total hours are not inferred from file size or an assumed night length. 时长口径：173.242 h（论文换算·明确范围；Common Sleep Data Pipeline Table 1: 20,789 retained 30-s epochs / 120 = 173.242 h; CSDP analysed cohort）</x:v>
       </x:c>
       <x:c r="S322" s="278"/>
-      <x:c r="T322" s="278"/>
+      <x:c r="T322" s="278" t="n">
+        <x:v>623670</x:v>
+      </x:c>
       <x:c r="U322" s="247" t="n">
         <x:v>25</x:v>
       </x:c>
@@ -21086,10 +21182,12 @@
         <x:v>02_Biometrics_and_Disease/Epilepsy_and_Abnormalities/HMS_Harmful_Brain_Activity_Classification</x:v>
       </x:c>
       <x:c r="R327" s="257" t="str">
-        <x:v>官方数据存在，但需申请、签署协议或获得权限</x:v>
+        <x:v>官方数据存在，但需申请、签署协议或获得权限 时长口径：390.16 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S327" s="257"/>
-      <x:c r="T327" s="257"/>
+      <x:c r="T327" s="257" t="n">
+        <x:v>1404576</x:v>
+      </x:c>
       <x:c r="U327" s="213"/>
     </x:row>
     <x:row r="328" ht="60" customHeight="1">
@@ -21145,10 +21243,12 @@
         <x:v>02_Biometrics_and_Disease/Epilepsy_and_Abnormalities/Interictal_Epileptiform_Discharge_EEG_Dataset</x:v>
       </x:c>
       <x:c r="R328" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号；2026-08-04去重：EEG-0019, EEG-0038并入EEG-0016（Figshare article 28069568）</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号；2026-08-04去重：EEG-0019, EEG-0038并入EEG-0016（Figshare article 28069568） 时长口径：28.242 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S328" s="275"/>
-      <x:c r="T328" s="275"/>
+      <x:c r="T328" s="275" t="n">
+        <x:v>101670</x:v>
+      </x:c>
       <x:c r="U328" s="276"/>
     </x:row>
     <x:row r="329" ht="60" customHeight="1">
@@ -21695,10 +21795,12 @@
         <x:v>02_Biometrics_and_Disease/Neurodegenerative_Disorders/APAVA</x:v>
       </x:c>
       <x:c r="R338" s="275" t="str">
-        <x:v>官方数据存在，但需申请、签署协议或获得权限</x:v>
+        <x:v>官方数据存在，但需申请、签署协议或获得权限 时长口径：0.921 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S338" s="275"/>
-      <x:c r="T338" s="275"/>
+      <x:c r="T338" s="275" t="n">
+        <x:v>3315</x:v>
+      </x:c>
       <x:c r="U338" s="276"/>
     </x:row>
     <x:row r="339" ht="60" customHeight="1">
@@ -21807,10 +21909,12 @@
         <x:v>02_Biometrics_and_Disease/Mental_and_Developmental_Disorders/Adult_ADHD_EEG</x:v>
       </x:c>
       <x:c r="R340" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号；2026-08-04去重：EEG-0049并入EEG-0048（Mendeley dataset 6k4g25fhzg）</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号；2026-08-04去重：EEG-0049并入EEG-0048（Mendeley dataset 6k4g25fhzg） 时长口径：7.111 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S340" s="275"/>
-      <x:c r="T340" s="275"/>
+      <x:c r="T340" s="275" t="n">
+        <x:v>25600</x:v>
+      </x:c>
       <x:c r="U340" s="276"/>
     </x:row>
     <x:row r="341" ht="60" customHeight="1">
@@ -21917,10 +22021,12 @@
         <x:v>02_Biometrics_and_Disease/Mental_and_Developmental_Disorders/EEG_in_schizophrenia</x:v>
       </x:c>
       <x:c r="R342" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：8.018 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S342" s="275"/>
-      <x:c r="T342" s="275"/>
+      <x:c r="T342" s="275" t="n">
+        <x:v>28863</x:v>
+      </x:c>
       <x:c r="U342" s="276"/>
     </x:row>
     <x:row r="343" ht="60" customHeight="1">
@@ -22027,10 +22133,12 @@
         <x:v>02_Biometrics_and_Disease/Mental_and_Developmental_Disorders/Schizophrenia-81</x:v>
       </x:c>
       <x:c r="R344" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：9.606 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S344" s="275"/>
-      <x:c r="T344" s="275"/>
+      <x:c r="T344" s="275" t="n">
+        <x:v>34581</x:v>
+      </x:c>
       <x:c r="U344" s="276"/>
     </x:row>
     <x:row r="345" ht="60" customHeight="1">
@@ -22082,10 +22190,12 @@
         <x:v>02_Biometrics_and_Disease/Mental_and_Developmental_Disorders/TDBRAIN</x:v>
       </x:c>
       <x:c r="R345" s="257" t="str">
-        <x:v>官方数据存在，但需申请、签署协议或获得权限</x:v>
+        <x:v>官方数据存在，但需申请、签署协议或获得权限 时长口径：120.516 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S345" s="257"/>
-      <x:c r="T345" s="257"/>
+      <x:c r="T345" s="257" t="n">
+        <x:v>433859</x:v>
+      </x:c>
       <x:c r="U345" s="213"/>
     </x:row>
     <x:row r="346" ht="60" customHeight="1">
@@ -22139,10 +22249,12 @@
         <x:v>02_Biometrics_and_Disease/Neurological_Disorders/ALS_Eye-tracking_Spelling_EEG_Dataset</x:v>
       </x:c>
       <x:c r="R346" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：267.145 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S346" s="275"/>
-      <x:c r="T346" s="275"/>
+      <x:c r="T346" s="275" t="n">
+        <x:v>961721.89359996</x:v>
+      </x:c>
       <x:c r="U346" s="276"/>
     </x:row>
     <x:row r="347" ht="60" customHeight="1">
@@ -22194,10 +22306,12 @@
         <x:v>02_Biometrics_and_Disease/Neurological_Disorders/BNCI_006-2014_SCP_training_in_stroke</x:v>
       </x:c>
       <x:c r="R347" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：21.876 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S347" s="257"/>
-      <x:c r="T347" s="257"/>
+      <x:c r="T347" s="257" t="n">
+        <x:v>78752</x:v>
+      </x:c>
       <x:c r="U347" s="213"/>
     </x:row>
     <x:row r="348" ht="60" customHeight="1">
@@ -22306,10 +22420,12 @@
         <x:v>02_Biometrics_and_Disease/Neurological_Disorders/MESA_Sleep</x:v>
       </x:c>
       <x:c r="R349" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：21,721.175 h（论文换算·明确范围；Common Sleep Data Pipeline Table 1: 2,606,541 retained 30-s epochs / 120 = 21721.175 h; CSDP analysed cohort）</x:v>
       </x:c>
       <x:c r="S349" s="257"/>
-      <x:c r="T349" s="257"/>
+      <x:c r="T349" s="257" t="n">
+        <x:v>78196230</x:v>
+      </x:c>
       <x:c r="U349" s="213"/>
     </x:row>
     <x:row r="350" ht="60" customHeight="1">
@@ -22473,10 +22589,12 @@
         <x:v>02_Biometrics_and_Disease/Neurological_Disorders/Tinnitus_Acoustic_Therapy_EEG_Database</x:v>
       </x:c>
       <x:c r="R352" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号；2026-08-04去重：EEG-0099, EEG-0315并入EEG-0098（Mendeley dataset kj443jc4yc）</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号；2026-08-04去重：EEG-0099, EEG-0315并入EEG-0098（Mendeley dataset kj443jc4yc） 时长口径：8.41 h（文件审计·部分范围；ACTUAL_DOWNLOADED_SCOPE_PARTIAL）</x:v>
       </x:c>
       <x:c r="S352" s="275"/>
-      <x:c r="T352" s="275"/>
+      <x:c r="T352" s="275" t="n">
+        <x:v>30276</x:v>
+      </x:c>
       <x:c r="U352" s="276"/>
     </x:row>
     <x:row r="353" ht="60" customHeight="1">
@@ -22803,10 +22921,12 @@
         <x:v>03_Consciousness_and_State/Sleep_Staging/CCSHS</x:v>
       </x:c>
       <x:c r="R358" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：5,761.683 h（论文换算·明确范围；Common Sleep Data Pipeline Table 1: 691,402 retained 30-s epochs / 120 = 5761.683 h; CSDP analysed cohort）</x:v>
       </x:c>
       <x:c r="S358" s="275"/>
-      <x:c r="T358" s="275"/>
+      <x:c r="T358" s="275" t="n">
+        <x:v>20742060</x:v>
+      </x:c>
       <x:c r="U358" s="276"/>
     </x:row>
     <x:row r="359" ht="60" customHeight="1">
@@ -22860,10 +22980,12 @@
         <x:v>03_Consciousness_and_State/Sleep_Staging/CFS</x:v>
       </x:c>
       <x:c r="R359" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：7,218.517 h（论文换算·明确范围；Common Sleep Data Pipeline Table 1: 866,222 retained 30-s epochs / 120 = 7218.517 h; CSDP analysed cohort）</x:v>
       </x:c>
       <x:c r="S359" s="257"/>
-      <x:c r="T359" s="257"/>
+      <x:c r="T359" s="257" t="n">
+        <x:v>25986660</x:v>
+      </x:c>
       <x:c r="U359" s="213"/>
     </x:row>
     <x:row r="360" ht="60" customHeight="1">
@@ -22915,10 +23037,12 @@
         <x:v>03_Consciousness_and_State/Sleep_Staging/CHAT</x:v>
       </x:c>
       <x:c r="R360" s="275" t="str">
-        <x:v>官方数据存在，但需申请、签署协议或获得权限</x:v>
+        <x:v>官方数据存在，但需申请、签署协议或获得权限 时长口径：16,319.508 h（论文换算·明确范围；Common Sleep Data Pipeline Table 1: 1,958,341 retained 30-s epochs / 120 = 16319.508 h; CSDP analysed cohort）</x:v>
       </x:c>
       <x:c r="S360" s="275"/>
-      <x:c r="T360" s="275"/>
+      <x:c r="T360" s="275" t="n">
+        <x:v>58750230</x:v>
+      </x:c>
       <x:c r="U360" s="276"/>
     </x:row>
     <x:row r="361" ht="60" customHeight="1">
@@ -23027,10 +23151,12 @@
         <x:v>03_Consciousness_and_State/Sleep_Staging/ISRUC-Sleep</x:v>
       </x:c>
       <x:c r="R362" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：777.75 h（论文换算·明确范围；Common Sleep Data Pipeline Table 1: 93,330 retained 30-s epochs / 120 = 777.750 h; CSDP ISRUC groups 1-3 analysed subset）</x:v>
       </x:c>
       <x:c r="S362" s="275"/>
-      <x:c r="T362" s="275"/>
+      <x:c r="T362" s="275" t="n">
+        <x:v>2799900</x:v>
+      </x:c>
       <x:c r="U362" s="276"/>
     </x:row>
     <x:row r="363" ht="60" customHeight="1">
@@ -23082,10 +23208,12 @@
         <x:v>03_Consciousness_and_State/Sleep_Staging/MASS</x:v>
       </x:c>
       <x:c r="R363" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：873.033 h（论文换算·明确范围；Common Sleep Data Pipeline Table 1: 104,764 retained 30-s epochs / 120 = 873.033 h; CSDP MASS cohorts 1 and 3 analysed subset）</x:v>
       </x:c>
       <x:c r="S363" s="257"/>
-      <x:c r="T363" s="257"/>
+      <x:c r="T363" s="257" t="n">
+        <x:v>3142920</x:v>
+      </x:c>
       <x:c r="U363" s="213"/>
     </x:row>
     <x:row r="364" ht="60" customHeight="1">
@@ -23357,10 +23485,12 @@
         <x:v>03_Consciousness_and_State/Sleep_Staging/MrOS_Sleep</x:v>
       </x:c>
       <x:c r="R368" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：44,987.817 h（论文换算·明确范围；Common Sleep Data Pipeline Table 1: 5,398,538 retained 30-s epochs / 120 = 44987.817 h; CSDP analysed cohort including longitudinal records）</x:v>
       </x:c>
       <x:c r="S368" s="275"/>
-      <x:c r="T368" s="275"/>
+      <x:c r="T368" s="275" t="n">
+        <x:v>161956140</x:v>
+      </x:c>
       <x:c r="U368" s="276"/>
     </x:row>
     <x:row r="369" ht="60" customHeight="1">
@@ -23467,10 +23597,12 @@
         <x:v>03_Consciousness_and_State/Sleep_Staging/SHHS</x:v>
       </x:c>
       <x:c r="R370" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：75,466.425 h（论文换算·明确范围；Common Sleep Data Pipeline Table 1: 9,055,971 retained 30-s epochs / 120 = 75466.425 h; CSDP analysed cohort）</x:v>
       </x:c>
       <x:c r="S370" s="275"/>
-      <x:c r="T370" s="275"/>
+      <x:c r="T370" s="275" t="n">
+        <x:v>271679130</x:v>
+      </x:c>
       <x:c r="U370" s="276"/>
     </x:row>
     <x:row r="371" ht="60" customHeight="1">
@@ -23522,10 +23654,12 @@
         <x:v>03_Consciousness_and_State/Sleep_Staging/SOF</x:v>
       </x:c>
       <x:c r="R371" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：4,514.133 h（论文换算·明确范围；Common Sleep Data Pipeline Table 1: 541,696 retained 30-s epochs / 120 = 4514.133 h; CSDP analysed cohort）</x:v>
       </x:c>
       <x:c r="S371" s="257"/>
-      <x:c r="T371" s="257"/>
+      <x:c r="T371" s="257" t="n">
+        <x:v>16250880</x:v>
+      </x:c>
       <x:c r="U371" s="213"/>
     </x:row>
     <x:row r="372" ht="60" customHeight="1">
@@ -27751,10 +27885,12 @@
         <x:v>02_Biometrics_and_Disease/Epilepsy_and_Abnormalities/Bonn_EEG_Seizure_Dataset</x:v>
       </x:c>
       <x:c r="R447" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号；2026-08-04去重：EEG-0037并入EEG-0008（Official University of Bonn landing page and Andrzejak 2001 corpus identity）</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号；2026-08-04去重：EEG-0037并入EEG-0008（Official University of Bonn landing page and Andrzejak 2001 corpus identity） 时长口径：3.278 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S447" s="257"/>
-      <x:c r="T447" s="257"/>
+      <x:c r="T447" s="257" t="n">
+        <x:v>11799.435516387304</x:v>
+      </x:c>
       <x:c r="U447" s="213"/>
     </x:row>
     <x:row r="448" ht="60" customHeight="1">
@@ -27808,10 +27944,12 @@
         <x:v>02_Biometrics_and_Disease/Neurodegenerative_Disorders/AD-Auditory</x:v>
       </x:c>
       <x:c r="R448" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：5.203 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S448" s="275"/>
-      <x:c r="T448" s="275"/>
+      <x:c r="T448" s="275" t="n">
+        <x:v>18730</x:v>
+      </x:c>
       <x:c r="U448" s="276"/>
     </x:row>
     <x:row r="449" ht="60" customHeight="1">
@@ -27865,10 +28003,12 @@
         <x:v>02_Biometrics_and_Disease/Neurodegenerative_Disorders/Dementia_Photo-stimulation_Open-eyes_EEG</x:v>
       </x:c>
       <x:c r="R449" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：14.963 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S449" s="257"/>
-      <x:c r="T449" s="257"/>
+      <x:c r="T449" s="257" t="n">
+        <x:v>53868.52800000001</x:v>
+      </x:c>
       <x:c r="U449" s="213"/>
     </x:row>
     <x:row r="450" ht="60" customHeight="1">
@@ -31337,10 +31477,12 @@
         <x:v>02_Biometrics_and_Disease/Development_and_Lifespan/Mind_in_Motion_Older_Adults_Walking_EEG</x:v>
       </x:c>
       <x:c r="R513" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：61.097 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S513" s="257"/>
-      <x:c r="T513" s="257"/>
+      <x:c r="T513" s="257" t="n">
+        <x:v>219948.69399999964</x:v>
+      </x:c>
       <x:c r="U513" s="213"/>
     </x:row>
     <x:row r="514" ht="60" customHeight="1">
@@ -31685,10 +31827,12 @@
         <x:v>02_Biometrics_and_Disease/Epilepsy_and_Abnormalities/OpenNeuro_ds003029_Epilepsy_iEEG_Multicenter</x:v>
       </x:c>
       <x:c r="R519" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：7.958 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S519" s="257"/>
-      <x:c r="T519" s="257"/>
+      <x:c r="T519" s="257" t="n">
+        <x:v>28650.020424195773</x:v>
+      </x:c>
       <x:c r="U519" s="213"/>
     </x:row>
     <x:row r="520" ht="60" customHeight="1">
@@ -31740,10 +31884,12 @@
         <x:v>02_Biometrics_and_Disease/Neurological_Disorders/UNMDataset</x:v>
       </x:c>
       <x:c r="R520" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：1.466 h（文件审计·部分范围；ACTUAL_DOWNLOADED_SCOPE_PARTIAL）</x:v>
       </x:c>
       <x:c r="S520" s="275"/>
-      <x:c r="T520" s="275"/>
+      <x:c r="T520" s="275" t="n">
+        <x:v>5277.6</x:v>
+      </x:c>
       <x:c r="U520" s="276"/>
     </x:row>
     <x:row r="521" ht="60" customHeight="1">
@@ -32394,10 +32540,12 @@
         <x:v>02_Biometrics_and_Disease/Epilepsy_and_Abnormalities/HUP_iEEG_Epilepsy_Dataset</x:v>
       </x:c>
       <x:c r="R532" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：49.769 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S532" s="275"/>
-      <x:c r="T532" s="275"/>
+      <x:c r="T532" s="275" t="n">
+        <x:v>179170</x:v>
+      </x:c>
       <x:c r="U532" s="276"/>
     </x:row>
     <x:row r="533" ht="60" customHeight="1">
@@ -32449,10 +32597,12 @@
         <x:v>02_Biometrics_and_Disease/Epilepsy_and_Abnormalities/Kaggle_UPenn_and_Mayo_Clinic_Seizure_Detection</x:v>
       </x:c>
       <x:c r="R533" s="257" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：16.35 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S533" s="257"/>
-      <x:c r="T533" s="257"/>
+      <x:c r="T533" s="257" t="n">
+        <x:v>58860.698923904565</x:v>
+      </x:c>
       <x:c r="U533" s="213"/>
     </x:row>
     <x:row r="534" ht="60" customHeight="1">
@@ -32504,10 +32654,12 @@
         <x:v>03_Consciousness_and_State/Sleep_Staging/ABC</x:v>
       </x:c>
       <x:c r="R534" s="275" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：1,109.175 h（论文换算·明确范围；Common Sleep Data Pipeline Table 1: 133,101 retained 30-s epochs / 120 = 1109.175 h; CSDP analysed cohort）</x:v>
       </x:c>
       <x:c r="S534" s="275"/>
-      <x:c r="T534" s="275"/>
+      <x:c r="T534" s="275" t="n">
+        <x:v>3993030</x:v>
+      </x:c>
       <x:c r="U534" s="276"/>
     </x:row>
     <x:row r="535" ht="60" customHeight="1">
@@ -32559,10 +32711,12 @@
         <x:v>03_Consciousness_and_State/Sleep_Staging/HomePAP</x:v>
       </x:c>
       <x:c r="R535" s="257" t="str">
-        <x:v>官方数据存在，但需申请、签署协议或获得权限</x:v>
+        <x:v>官方数据存在，但需申请、签署协议或获得权限 时长口径：1,928.633 h（论文换算·明确范围；Common Sleep Data Pipeline Table 1: 231,436 retained 30-s epochs / 120 = 1928.633 h; CSDP subset (247 records; catalog release is wider)）</x:v>
       </x:c>
       <x:c r="S535" s="257"/>
-      <x:c r="T535" s="257"/>
+      <x:c r="T535" s="257" t="n">
+        <x:v>6943080</x:v>
+      </x:c>
       <x:c r="U535" s="213"/>
     </x:row>
     <x:row r="536" ht="60" customHeight="1">
@@ -33164,10 +33318,12 @@
         <x:v>02_Biometrics_and_Disease/Epilepsy_and_Abnormalities/American_Epilepsy_Society_Seizure_Prediction_Challenge</x:v>
       </x:c>
       <x:c r="R546" s="280" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：1,333.667 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S546" s="280"/>
-      <x:c r="T546" s="280"/>
+      <x:c r="T546" s="280" t="n">
+        <x:v>4801200</x:v>
+      </x:c>
       <x:c r="U546" s="281"/>
     </x:row>
     <x:row r="547">
@@ -33274,7 +33430,7 @@
         <x:v>03_Consciousness_and_State/Sleep_Staging/ASCERTAIN</x:v>
       </x:c>
       <x:c r="R548" s="280" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号 分类复核：ASCERTAIN is an affect/personality experiment, not a sleep or clinical cohort. 分类复核：ASCERTAIN is an affect/personality experiment, not a sleep or clinical cohort. 分类复核：ASCERTAIN is an affect/personality experiment, not a sleep or clinical cohort. 分类复核：ASCERTAIN is an affect/personality experiment, not a sleep or clinical cohort.</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 分类复核：ASCERTAIN is an affect/personality experiment, not a sleep or clinical cohort. 分类复核：ASCERTAIN is an affect/personality experiment, not a sleep or clinical cohort. 分类复核：ASCERTAIN is an affect/personality experiment, not a sleep or clinical cohort. 分类复核：ASCERTAIN is an affect/personality experiment, not a sleep or clinical cohort. 分类复核：ASCERTAIN is an affect/personality experiment, not a sleep or clinical cohort.</x:v>
       </x:c>
       <x:c r="S548" s="280"/>
       <x:c r="T548" s="280"/>
@@ -33916,10 +34072,12 @@
         <x:v>02_Biometrics_and_Disease/Epilepsy_and_Abnormalities/BEED</x:v>
       </x:c>
       <x:c r="R560" s="280" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：88.889 h（论文/官网记录；DOCUMENTED_PROTOCOL）</x:v>
       </x:c>
       <x:c r="S560" s="280"/>
-      <x:c r="T560" s="280"/>
+      <x:c r="T560" s="280" t="n">
+        <x:v>320000</x:v>
+      </x:c>
       <x:c r="U560" s="281"/>
     </x:row>
     <x:row r="561">
@@ -34026,10 +34184,12 @@
         <x:v>02_Biometrics_and_Disease/Development_and_Lifespan/MIPDB</x:v>
       </x:c>
       <x:c r="R562" s="280" t="str">
-        <x:v>存在公开仓库、官方入口或稳定数据访问号</x:v>
+        <x:v>存在公开仓库、官方入口或稳定数据访问号 时长口径：104.05 h（文件审计·精确；ACTUAL_DOWNLOADED_SCOPE_EXACT）</x:v>
       </x:c>
       <x:c r="S562" s="280"/>
-      <x:c r="T562" s="280"/>
+      <x:c r="T562" s="280" t="n">
+        <x:v>374580.18799999997</x:v>
+      </x:c>
       <x:c r="U562" s="281"/>
     </x:row>
     <x:row r="563">
@@ -34090,7 +34250,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R334d792b93114e18"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6355cae59084888"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34212,19 +34372,19 @@
         <x:v>2026-08-23</x:v>
       </x:c>
       <x:c r="B6" s="400" t="str">
-        <x:v>AUDIT</x:v>
+        <x:v>DURATION</x:v>
       </x:c>
       <x:c r="C6" s="400" t="str">
-        <x:v>疾病/健康 146 项</x:v>
+        <x:v>93 catalog units</x:v>
       </x:c>
       <x:c r="D6" s="400" t="str">
-        <x:v>确认服务器完成 80 项、独立 raw 73 项、精确时长 57 项。</x:v>
+        <x:v>将疾病/健康文件审计和论文时长回填总表；其中 62 项有文件/下载范围审计，31 项仅用论文或官网范围。</x:v>
       </x:c>
       <x:c r="E6" s="400" t="str">
-        <x:v>SeaWulf VPN 只读快照</x:v>
+        <x:v>Common Sleep Data Pipeline Table 1；本地 EDF/数据发布审计</x:v>
       </x:c>
       <x:c r="F6" s="401" t="str">
-        <x:v>未改服务器文件</x:v>
+        <x:v>无</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="54" customHeight="1">
@@ -34232,19 +34392,19 @@
         <x:v>2026-08-23</x:v>
       </x:c>
       <x:c r="B7" s="257" t="str">
-        <x:v>ACCESS</x:v>
+        <x:v>AUDIT</x:v>
       </x:c>
       <x:c r="C7" s="257" t="str">
-        <x:v>SeizeIT</x:v>
+        <x:v>疾病/健康 146 项</x:v>
       </x:c>
       <x:c r="D7" s="257" t="str">
-        <x:v>SeizeIT2（EEG-0031）已下载并审计 11,626.25 h；SeizeIT1 因官方不可获取而舍弃。</x:v>
+        <x:v>确认服务器完成 80 项、独立 raw 73 项、精确时长 57 项。</x:v>
       </x:c>
       <x:c r="E7" s="257" t="str">
-        <x:v>OpenNeuro ds005873 + KU Leuven SeizeIT1 record</x:v>
+        <x:v>SeaWulf VPN 只读快照</x:v>
       </x:c>
       <x:c r="F7" s="213" t="str">
-        <x:v>避免重复下载</x:v>
+        <x:v>未改服务器文件</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="54" customHeight="1">
@@ -34255,16 +34415,16 @@
         <x:v>ACCESS</x:v>
       </x:c>
       <x:c r="C8" s="400" t="str">
-        <x:v>EEG-0093 / EEG-0122</x:v>
+        <x:v>SeizeIT</x:v>
       </x:c>
       <x:c r="D8" s="400" t="str">
-        <x:v>PD-Mortality 更新为 OpenNeuro ds007020；DOD-H 更新为官方 Zenodo:15900394，并按健康志愿者队列改归 Health。</x:v>
+        <x:v>SeizeIT2（EEG-0031）已下载并审计 11,626.25 h；SeizeIT1 因官方不可获取而舍弃。</x:v>
       </x:c>
       <x:c r="E8" s="400" t="str">
-        <x:v>OpenNeuro ds007020；DOI:10.5281/zenodo.15900394</x:v>
+        <x:v>OpenNeuro ds005873 + KU Leuven SeizeIT1 record</x:v>
       </x:c>
       <x:c r="F8" s="401" t="str">
-        <x:v>两项已下载</x:v>
+        <x:v>避免重复下载</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="54" customHeight="1">
@@ -34275,16 +34435,16 @@
         <x:v>ACCESS</x:v>
       </x:c>
       <x:c r="C9" s="257" t="str">
-        <x:v>MODMA / CHBMP</x:v>
+        <x:v>EEG-0093 / EEG-0122</x:v>
       </x:c>
       <x:c r="D9" s="257" t="str">
-        <x:v>MODMA ID 13/14/17 已获批，入口双端复测恢复并需重新登录；CHBMP 已获批，首批 32/250 raw sessions 下载并完成 EDF 头审计。</x:v>
+        <x:v>PD-Mortality 更新为 OpenNeuro ds007020；DOD-H 更新为官方 Zenodo:15900394，并按健康志愿者队列改归 Health。</x:v>
       </x:c>
       <x:c r="E9" s="257" t="str">
-        <x:v>MODMA 个人授权；CHBMP LORIS</x:v>
+        <x:v>OpenNeuro ds007020；DOI:10.5281/zenodo.15900394</x:v>
       </x:c>
       <x:c r="F9" s="213" t="str">
-        <x:v>CHBMP 新增 32 EDF / 10.9689 h</x:v>
+        <x:v>两项已下载</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -34292,19 +34452,19 @@
         <x:v>2026-08-23</x:v>
       </x:c>
       <x:c r="B10" s="328" t="str">
-        <x:v>DOWNLOAD</x:v>
+        <x:v>ACCESS</x:v>
       </x:c>
       <x:c r="C10" s="328" t="str">
-        <x:v>19 public units</x:v>
+        <x:v>MODMA / CHBMP</x:v>
       </x:c>
       <x:c r="D10" s="328" t="str">
-        <x:v>优先疾病/Health：Albrecht2019、Gruendler2009、Singh2020、Singh2021、PD-Mortality、DOD-H 已完成；HMC、UCDDB 下载中；其余 11 项暂不启动以保留预处理空间。</x:v>
+        <x:v>MODMA ID 13/14/17 已获批，入口双端复测恢复并需重新登录；CHBMP 已获批，首批 32/250 raw sessions 下载并完成 EDF 头审计。</x:v>
       </x:c>
       <x:c r="E10" s="328" t="str">
-        <x:v>服务器 .download_complete 标记与 Slurm 2133731</x:v>
+        <x:v>MODMA 个人授权；CHBMP LORIS</x:v>
       </x:c>
       <x:c r="F10" s="329" t="str">
-        <x:v>6 完成 / 2 下载中</x:v>
+        <x:v>CHBMP 新增 32 EDF / 10.9689 h</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -34312,19 +34472,19 @@
         <x:v>2026-08-23</x:v>
       </x:c>
       <x:c r="B11" s="259" t="str">
-        <x:v>ACCESS</x:v>
+        <x:v>DOWNLOAD</x:v>
       </x:c>
       <x:c r="C11" s="259" t="str">
-        <x:v>MORGOTH PSG</x:v>
+        <x:v>19 public units</x:v>
       </x:c>
       <x:c r="D11" s="259" t="str">
-        <x:v>4 个 PSG 子集并入已提交的 MORGOTH credentialed-access 申请。</x:v>
+        <x:v>优先疾病/Health：Albrecht2019、Gruendler2009、Singh2020、Singh2021、PD-Mortality、DOD-H 已完成；HMC、UCDDB 下载中；其余 11 项暂不启动以保留预处理空间。</x:v>
       </x:c>
       <x:c r="E11" s="259" t="str">
-        <x:v>BDSP MORGOTH 1.0</x:v>
+        <x:v>服务器 .download_complete 标记与 Slurm 2133731</x:v>
       </x:c>
       <x:c r="F11" s="215" t="str">
-        <x:v>等待授权</x:v>
+        <x:v>6 完成 / 2 下载中</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -34332,45 +34492,65 @@
         <x:v>2026-08-23</x:v>
       </x:c>
       <x:c r="B12" s="328" t="str">
+        <x:v>ACCESS</x:v>
+      </x:c>
+      <x:c r="C12" s="328" t="str">
+        <x:v>MORGOTH PSG</x:v>
+      </x:c>
+      <x:c r="D12" s="328" t="str">
+        <x:v>4 个 PSG 子集并入已提交的 MORGOTH credentialed-access 申请。</x:v>
+      </x:c>
+      <x:c r="E12" s="328" t="str">
+        <x:v>BDSP MORGOTH 1.0</x:v>
+      </x:c>
+      <x:c r="F12" s="329" t="str">
+        <x:v>等待授权</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="226" t="str">
+        <x:v>2026-08-23</x:v>
+      </x:c>
+      <x:c r="B13" s="259" t="str">
         <x:v>QUEUE</x:v>
       </x:c>
-      <x:c r="C12" s="328" t="str">
+      <x:c r="C13" s="259" t="str">
         <x:v>62 actionable</x:v>
       </x:c>
-      <x:c r="D12" s="328" t="str">
+      <x:c r="D13" s="259" t="str">
         <x:v>正式需申请 41 项：已申请 19 项，尚需申请 22 项；另有 4 项舍弃。</x:v>
       </x:c>
-      <x:c r="E12" s="328" t="str">
+      <x:c r="E13" s="259" t="str">
         <x:v>逐项官方访问入口复核</x:v>
       </x:c>
-      <x:c r="F12" s="329" t="str">
+      <x:c r="F13" s="215" t="str">
         <x:v>更新执行队列</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="227" t="str">
+    <x:row r="14">
+      <x:c r="A14" s="234" t="str">
         <x:v>2026-08-23</x:v>
       </x:c>
-      <x:c r="B13" s="270" t="str">
+      <x:c r="B14" s="359" t="str">
         <x:v>FORMAT</x:v>
       </x:c>
-      <x:c r="C13" s="270" t="str">
+      <x:c r="C14" s="359" t="str">
         <x:v>Workbook</x:v>
       </x:c>
-      <x:c r="D13" s="270" t="str">
+      <x:c r="D14" s="359" t="str">
         <x:v>公开下载工作簿精简为 README、最终唯一下载清单、修订记录 3 张表。</x:v>
       </x:c>
-      <x:c r="E13" s="270" t="str">
+      <x:c r="E14" s="359" t="str">
         <x:v>用户要求</x:v>
       </x:c>
-      <x:c r="F13" s="228" t="str">
+      <x:c r="F14" s="360" t="str">
         <x:v>无</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8b134f152fa43e5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea276086854f4c22"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Mark MODMA download complete across catalog
</commit_message>
<xml_diff>
--- a/EEG_healthcare_disease_catalog_20260823.xlsx
+++ b/EEG_healthcare_disease_catalog_20260823.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R393821410cf64387"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最终唯一下载清单" sheetId="2" r:id="Rb816959c60e94aca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="修订记录" sheetId="8" r:id="Rfbac854391d94f54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rc7d0a1bb615048a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="最终唯一下载清单" sheetId="2" r:id="R245eb5ccaf044b69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="修订记录" sheetId="8" r:id="R2c7f7906470a4822"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1589,7 +1589,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="RevisionLog20260823" displayName="RevisionLog20260823" ref="A1:F15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="RevisionLog20260823" displayName="RevisionLog20260823" ref="A1:F16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Change type"/>
@@ -1812,7 +1812,7 @@
         <x:v>修订日期</x:v>
       </x:c>
       <x:c r="B2" s="211" t="str">
-        <x:v>2026-08-23</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
@@ -1852,7 +1852,7 @@
         <x:v>服务器完成目录</x:v>
       </x:c>
       <x:c r="B7" s="247" t="str">
-        <x:v>80 units（含 TUH 重叠与非 raw 排除项）</x:v>
+        <x:v>81 units（含 TUH 重叠与非 raw 排除项）</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
@@ -1860,7 +1860,7 @@
         <x:v>独立 raw 已获取</x:v>
       </x:c>
       <x:c r="B8" s="247" t="str">
-        <x:v>73 units（疾病 59 / Health 14）</x:v>
+        <x:v>74 units（疾病 60 / Health 14）</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="34" customHeight="1">
@@ -1884,7 +1884,7 @@
         <x:v>下载执行队列</x:v>
       </x:c>
       <x:c r="B11" s="247" t="str">
-        <x:v>63 个仍可推进；4 个舍弃但保留目录证据</x:v>
+        <x:v>62 个仍可推进；4 个舍弃但保留目录证据</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="58" customHeight="1">
@@ -1900,7 +1900,7 @@
         <x:v>直接推进</x:v>
       </x:c>
       <x:c r="B13" s="213" t="str">
-        <x:v>2 个下载中；12 个可直接下载；3 个只需登录；5 个需人工确认文件入口</x:v>
+        <x:v>2 个下载中；12 个可直接下载；2 个只需登录；5 个需人工确认文件入口</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="58" customHeight="1">
@@ -1956,7 +1956,7 @@
         <x:v>口径提醒</x:v>
       </x:c>
       <x:c r="B20" s="215" t="str">
-        <x:v>73 是服务器目录与独立 raw 获取口径；57 / 43627.8 h 是已有时长审计口径；346490.7 h 是来源覆盖下界估计，三者不可混写。</x:v>
+        <x:v>74 是服务器目录与独立 raw 获取口径；57 / 43627.8 h 是已有时长审计口径；346490.7 h 是来源覆盖下界估计，三者不可混写。</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -2004,7 +2004,7 @@
         <x:v>已获批访问</x:v>
       </x:c>
       <x:c r="B26" s="215" t="str">
-        <x:v>CHBMP：32/250 raw sessions 已下载并审计 10.9689 h；MODMA：ID 13/14/17 已获批，入口双端复测恢复，需重新登录。</x:v>
+        <x:v>CHBMP：32/250 raw sessions 已下载并审计 10.9689 h；MODMA：ID 13/14/17 三个 ZIP 已完整下载（7.59 GB），其中 ID 14/17 匹配官网 MD5，ID 13 通过服务器长度与 60/60 ZIP CRC。</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -23306,7 +23306,7 @@
         <x:v>02_Biometrics_and_Disease/Mental_and_Developmental_Disorders/MODMA</x:v>
       </x:c>
       <x:c r="R364" s="275" t="str">
-        <x:v>官方数据存在，但需申请、签署协议或获得权限</x:v>
+        <x:v>官方数据存在，但需申请、签署协议或获得权限 2026-08-25 authenticated download complete: IDs 13/14/17, 7,593,313,997 bytes. ID 14/17 match the published MD5; ID 13 matches the current server size and passes all 60 ZIP CRCs while the published MD5 discrepancy is retained in the manifest.</x:v>
       </x:c>
       <x:c r="S364" s="275"/>
       <x:c r="T364" s="275"/>
@@ -34322,7 +34322,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ce41b95ae3b4648"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28ec2f4819634423"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34490,7 +34490,7 @@
         <x:v>疾病/健康 147 项</x:v>
       </x:c>
       <x:c r="D8" s="403" t="str">
-        <x:v>确认服务器完成 80 项、独立 raw 73 项、精确时长 57 项。</x:v>
+        <x:v>确认服务器完成 81 项、独立 raw 74 项、精确时长 57 项。</x:v>
       </x:c>
       <x:c r="E8" s="403" t="str">
         <x:v>SeaWulf VPN 只读快照</x:v>
@@ -34550,7 +34550,7 @@
         <x:v>MODMA / CHBMP</x:v>
       </x:c>
       <x:c r="D11" s="259" t="str">
-        <x:v>MODMA ID 13/14/17 已获批，入口双端复测恢复并需重新登录；CHBMP 已获批，首批 32/250 raw sessions 下载并完成 EDF 头审计。</x:v>
+        <x:v>MODMA ID 13/14/17 已获批；CHBMP 已获批，首批 32/250 raw sessions 下载并完成 EDF 头审计。</x:v>
       </x:c>
       <x:c r="E11" s="259" t="str">
         <x:v>MODMA 个人授权；CHBMP LORIS</x:v>
@@ -34561,22 +34561,22 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="233" t="str">
-        <x:v>2026-08-23</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="B12" s="334" t="str">
         <x:v>DOWNLOAD</x:v>
       </x:c>
       <x:c r="C12" s="334" t="str">
-        <x:v>19 public units</x:v>
+        <x:v>MODMA / EEG-0058</x:v>
       </x:c>
       <x:c r="D12" s="334" t="str">
-        <x:v>优先疾病/Health：Albrecht2019、Gruendler2009、Singh2020、Singh2021、PD-Mortality、DOD-H 已完成；HMC、UCDDB 下载中；其余 11 项暂不启动以保留预处理空间。</x:v>
+        <x:v>三个授权 ZIP 已完成，共 7,593,313,997 bytes；ID 14/17 与发布 MD5 一致，ID 13 当前服务器文件大小一致且 60/60 ZIP CRC 通过，发布 MD5 差异保留在 manifest。</x:v>
       </x:c>
       <x:c r="E12" s="334" t="str">
-        <x:v>服务器 .download_complete 标记与 Slurm 2133731</x:v>
+        <x:v>SeaWulf raw/download_manifest.json；全量 ZIP CRC 审计</x:v>
       </x:c>
       <x:c r="F12" s="335" t="str">
-        <x:v>6 完成 / 2 下载中</x:v>
+        <x:v>新增 .download_complete；标记已下载待时长审计</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -34584,19 +34584,19 @@
         <x:v>2026-08-23</x:v>
       </x:c>
       <x:c r="B13" s="259" t="str">
-        <x:v>ACCESS</x:v>
+        <x:v>DOWNLOAD</x:v>
       </x:c>
       <x:c r="C13" s="259" t="str">
-        <x:v>MORGOTH PSG</x:v>
+        <x:v>19 public units</x:v>
       </x:c>
       <x:c r="D13" s="259" t="str">
-        <x:v>4 个 PSG 子集并入已提交的 MORGOTH credentialed-access 申请。</x:v>
+        <x:v>优先疾病/Health：Albrecht2019、Gruendler2009、Singh2020、Singh2021、PD-Mortality、DOD-H 已完成；HMC、UCDDB 下载中；其余 11 项暂不启动以保留预处理空间。</x:v>
       </x:c>
       <x:c r="E13" s="259" t="str">
-        <x:v>BDSP MORGOTH 1.0</x:v>
+        <x:v>服务器 .download_complete 标记与 Slurm 2133731</x:v>
       </x:c>
       <x:c r="F13" s="215" t="str">
-        <x:v>等待授权</x:v>
+        <x:v>6 完成 / 2 下载中</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -34604,45 +34604,65 @@
         <x:v>2026-08-23</x:v>
       </x:c>
       <x:c r="B14" s="334" t="str">
+        <x:v>ACCESS</x:v>
+      </x:c>
+      <x:c r="C14" s="334" t="str">
+        <x:v>MORGOTH PSG</x:v>
+      </x:c>
+      <x:c r="D14" s="334" t="str">
+        <x:v>4 个 PSG 子集并入已提交的 MORGOTH credentialed-access 申请。</x:v>
+      </x:c>
+      <x:c r="E14" s="334" t="str">
+        <x:v>BDSP MORGOTH 1.0</x:v>
+      </x:c>
+      <x:c r="F14" s="335" t="str">
+        <x:v>等待授权</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="226" t="str">
+        <x:v>2026-08-23</x:v>
+      </x:c>
+      <x:c r="B15" s="259" t="str">
         <x:v>QUEUE</x:v>
       </x:c>
-      <x:c r="C14" s="334" t="str">
-        <x:v>63 actionable</x:v>
-      </x:c>
-      <x:c r="D14" s="334" t="str">
+      <x:c r="C15" s="259" t="str">
+        <x:v>62 actionable</x:v>
+      </x:c>
+      <x:c r="D15" s="259" t="str">
         <x:v>正式需申请 41 项：已申请 19 项，尚需申请 22 项；另有 4 项舍弃。</x:v>
       </x:c>
-      <x:c r="E14" s="334" t="str">
+      <x:c r="E15" s="259" t="str">
         <x:v>逐项官方访问入口复核</x:v>
       </x:c>
-      <x:c r="F14" s="335" t="str">
+      <x:c r="F15" s="215" t="str">
         <x:v>更新执行队列</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="227" t="str">
+    <x:row r="16">
+      <x:c r="A16" s="234" t="str">
         <x:v>2026-08-23</x:v>
       </x:c>
-      <x:c r="B15" s="270" t="str">
+      <x:c r="B16" s="336" t="str">
         <x:v>FORMAT</x:v>
       </x:c>
-      <x:c r="C15" s="270" t="str">
+      <x:c r="C16" s="336" t="str">
         <x:v>Workbook</x:v>
       </x:c>
-      <x:c r="D15" s="270" t="str">
+      <x:c r="D16" s="336" t="str">
         <x:v>公开下载工作簿精简为 README、最终唯一下载清单、修订记录 3 张表。</x:v>
       </x:c>
-      <x:c r="E15" s="270" t="str">
+      <x:c r="E16" s="336" t="str">
         <x:v>用户要求</x:v>
       </x:c>
-      <x:c r="F15" s="228" t="str">
+      <x:c r="F16" s="337" t="str">
         <x:v>无</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52c6b2bbac174d0a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70bc9bcb162f4e76"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>